<commit_message>
ignored the processed data
</commit_message>
<xml_diff>
--- a/data/processed/candidates.xlsx
+++ b/data/processed/candidates.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="354">
   <si>
     <t>place_id</t>
   </si>
@@ -49,15 +49,9 @@
     <t>google_maps_url</t>
   </si>
   <si>
-    <t>ChIJkaD3fMVQw0cR0Y-SgHCHlvw</t>
-  </si>
-  <si>
     <t>ChIJv8_dynU9w0cRPwuu4Hw6BCM</t>
   </si>
   <si>
-    <t>ChIJD_pZGNBQw0cRD-WANdpmDGk</t>
-  </si>
-  <si>
     <t>ChIJ6U6ntWgUw0cRZrq8q_ohqUU</t>
   </si>
   <si>
@@ -67,15 +61,12 @@
     <t>ChIJd92M2UBxw0cRcLC_XWtAw5M</t>
   </si>
   <si>
+    <t>ChIJcw76AERxw0cRCZ9UPLL7szA</t>
+  </si>
+  <si>
     <t>ChIJfXFDIWBxw0cRE9YYAtd17F4</t>
   </si>
   <si>
-    <t>ChIJcw76AERxw0cRCZ9UPLL7szA</t>
-  </si>
-  <si>
-    <t>ChIJO6D6ut1Qw0cRfRITh057Upg</t>
-  </si>
-  <si>
     <t>ChIJYdFddZ1nw0cRf0zN9IQqQ7Q</t>
   </si>
   <si>
@@ -85,12 +76,12 @@
     <t>ChIJ66An1k1xw0cRrkKcb_6Z488</t>
   </si>
   <si>
+    <t>ChIJl4CsVsF2w0cRytpeXShIbNE</t>
+  </si>
+  <si>
     <t>ChIJI46pG0dxw0cRIXbgTe31oZc</t>
   </si>
   <si>
-    <t>ChIJl4CsVsF2w0cRytpeXShIbNE</t>
-  </si>
-  <si>
     <t>ChIJvwaiZ1pxw0cRITmiV6KwtPw</t>
   </si>
   <si>
@@ -100,18 +91,36 @@
     <t>ChIJZ6VMYFdxw0cRfVoCvTscwOg</t>
   </si>
   <si>
+    <t>ChIJl8_4Z05xw0cRY8fapfMJrxc</t>
+  </si>
+  <si>
     <t>ChIJr82_7G1yw0cRebseGTV57d0</t>
   </si>
   <si>
-    <t>ChIJl8_4Z05xw0cRY8fapfMJrxc</t>
-  </si>
-  <si>
-    <t>ChIJocMKhOE6w0cRiwy8ypm_OLY</t>
-  </si>
-  <si>
     <t>ChIJD8S0YEdxw0cRfVs16dksyJQ</t>
   </si>
   <si>
+    <t>ChIJi-zbr0UQw0cRyBDtc11VPiE</t>
+  </si>
+  <si>
+    <t>ChIJyXZkekZxw0cRb9uqej8bxZY</t>
+  </si>
+  <si>
+    <t>ChIJs0g1-kZxw0cR46lPwxTdOpg</t>
+  </si>
+  <si>
+    <t>ChIJU1sJSUZxw0cRgmHC8o3MZwQ</t>
+  </si>
+  <si>
+    <t>ChIJ0X-9015xw0cRsPLuG79Kn4s</t>
+  </si>
+  <si>
+    <t>ChIJO5B6a0Zxw0cRCSaWrQEL7bE</t>
+  </si>
+  <si>
+    <t>ChIJW3OtxDlxw0cRM_nXQaujiBg</t>
+  </si>
+  <si>
     <t>ChIJmzeJyjnWwkcRCMoN538F2as</t>
   </si>
   <si>
@@ -133,9 +142,18 @@
     <t>ChIJCQOYnYjVwkcR6lYaR-xTg98</t>
   </si>
   <si>
+    <t>ChIJn9OLi97fwkcRN9zVioh1KUc</t>
+  </si>
+  <si>
     <t>ChIJGV-_vdfTwkcRX88cSrHGyf8</t>
   </si>
   <si>
+    <t>ChIJiXvXemrWwkcR1Th5LFqOW7s</t>
+  </si>
+  <si>
+    <t>ChIJb-2V4XYqw0cRcdf1yjoy0F8</t>
+  </si>
+  <si>
     <t>ChIJbx9ih_Aw3UcRoGOf2o5HMr4</t>
   </si>
   <si>
@@ -148,34 +166,16 @@
     <t>ChIJ1WAX4MM-3UcRMMlIwokR7OY</t>
   </si>
   <si>
+    <t>ChIJPdx5aSXbwkcRQhNCE1K7LD4</t>
+  </si>
+  <si>
     <t>ChIJ3d3K12fJwkcR0dksDPOE-LE</t>
   </si>
   <si>
     <t>ChIJI5GNfGfJwkcRkvhp-n7tsQo</t>
   </si>
   <si>
-    <t>ChIJe_MMnkYt3UcRc-auwbiNW0c</t>
-  </si>
-  <si>
-    <t>ChIJ-V0ngnRI3UcRxNYJAxiXTqM</t>
-  </si>
-  <si>
-    <t>ChIJV7YKDXUw3UcRFedUAMyku0M</t>
-  </si>
-  <si>
-    <t>ChIJs-JfFD-E50cRkks1dAfeD04</t>
-  </si>
-  <si>
-    <t>ChIJod-1BEeE50cRGEbTCldDiEk</t>
-  </si>
-  <si>
-    <t>ChIJKTehx0mE50cRRBnfjWRP2e8</t>
-  </si>
-  <si>
-    <t>ChIJGTko2DiE50cRmeo-Et037Rs</t>
-  </si>
-  <si>
-    <t>ChIJT7GmqkeE50cRjqo3SaXmEFs</t>
+    <t>ChIJMdnRjTG6wkcRhoM1KoA2Xl8</t>
   </si>
   <si>
     <t>ChIJdU5gH9dT3UcRL5zDVej010Y</t>
@@ -184,49 +184,61 @@
     <t>ChIJ2WXVuTBZ3UcRf0B-9mmdb1Q</t>
   </si>
   <si>
-    <t>ChIJ-W2FEpiG50cRVoTEf_6176I</t>
-  </si>
-  <si>
-    <t>ChIJY2VhcpGF50cRSy6NwjYOsPo</t>
-  </si>
-  <si>
-    <t>ChIJsRkGiICP50cR4y6APgUdWNA</t>
+    <t>ChIJz9Z6O4UA6EcRRbZGn3G3gbM</t>
+  </si>
+  <si>
+    <t>ChIJaYuwuJoA6EcRk7-jwtLVO8g</t>
+  </si>
+  <si>
+    <t>ChIJtTuE06D-50cR2--b95hIc8I</t>
+  </si>
+  <si>
+    <t>ChIJib4_kqMA6EcRD6sUNY4aftQ</t>
+  </si>
+  <si>
+    <t>ChIJaaZMOMPv50cRV7HwbArC9bQ</t>
+  </si>
+  <si>
+    <t>ChIJ81iJTsMC6EcRB7QQZNBe63c</t>
   </si>
   <si>
     <t>ChIJu9TW-YeM50cRWgv1BJZBEA0</t>
   </si>
   <si>
-    <t>ChIJT-FpWzaE50cR1O3LCiccUps</t>
-  </si>
-  <si>
-    <t>ChIJ866YABOJ50cR64ETj_MHZBM</t>
-  </si>
-  <si>
-    <t>ChIJG910IIOP50cRXrfJdLILZ2Y</t>
-  </si>
-  <si>
-    <t>ChIJvb4H_Rp-3UcR3lsWBx04w6U</t>
-  </si>
-  <si>
-    <t>ChIJQcUaDH-F50cRis_9pkrt7CY</t>
-  </si>
-  <si>
-    <t>ChIJ4SFseEiE50cReLJiUM2S_o8</t>
-  </si>
-  <si>
-    <t>ChIJmTVfja2F50cRk-m6tyEg5ic</t>
-  </si>
-  <si>
-    <t>ChIJhwejHDCE50cRyPI1ZjgtwAU</t>
-  </si>
-  <si>
-    <t>ChIJ8fgtIkqE50cRhFjeGhOUc-k</t>
-  </si>
-  <si>
-    <t>ChIJRfSU7kmE50cRZUAzMfzB-CU</t>
-  </si>
-  <si>
-    <t>ChIJcYYKwkuE50cRM00saJuEInU</t>
+    <t>ChIJxxW9nDpZ3UcRq2W4vQBjXdo</t>
+  </si>
+  <si>
+    <t>ChIJqbcdlZwA6EcRwvpe_YOrcIA</t>
+  </si>
+  <si>
+    <t>ChIJ1QnuayDn50cR2Dz4I-QJwz8</t>
+  </si>
+  <si>
+    <t>ChIJl5YJwavz50cRrswjHSVYqX4</t>
+  </si>
+  <si>
+    <t>ChIJA-D9f_rm50cR3alW2glvv0s</t>
+  </si>
+  <si>
+    <t>ChIJO4XZwNjm50cR7TkMIfUH8i0</t>
+  </si>
+  <si>
+    <t>ChIJf6fIWTBM3UcR481vvWP5QAk</t>
+  </si>
+  <si>
+    <t>ChIJ0b2ioiDn50cRSacFMQFo1gs</t>
+  </si>
+  <si>
+    <t>ChIJx0IhISND3UcRulMyFL2o8-A</t>
+  </si>
+  <si>
+    <t>ChIJZ5IoFBVV3UcRfzObqtmTFuw</t>
+  </si>
+  <si>
+    <t>ChIJEQnn8yLn50cRGCqPPfadcEk</t>
+  </si>
+  <si>
+    <t>ChIJVToX4xIO6EcRcQvXHvdfhpA</t>
   </si>
   <si>
     <t>ChIJ3fl0IYHW50cR_mvDeqFjsfs</t>
@@ -292,15 +304,9 @@
     <t>ChIJrVot9YPW50cRO0325Mfvbes</t>
   </si>
   <si>
-    <t>Duc De Bourgogne</t>
-  </si>
-  <si>
     <t>Restaurant Beukenhof Vichte</t>
   </si>
   <si>
-    <t>Verdi B&amp;B</t>
-  </si>
-  <si>
     <t>Hof van Cleve</t>
   </si>
   <si>
@@ -310,15 +316,12 @@
     <t>Korenlei Twee</t>
   </si>
   <si>
+    <t>Lucy Chang Gent</t>
+  </si>
+  <si>
     <t>Café Parti</t>
   </si>
   <si>
-    <t>Lucy Chang Gent</t>
-  </si>
-  <si>
-    <t>'t Bagientje</t>
-  </si>
-  <si>
     <t>'t Brigandje</t>
   </si>
   <si>
@@ -328,12 +331,12 @@
     <t>faim fatale</t>
   </si>
   <si>
+    <t>LAGO Gent Rozebroeken</t>
+  </si>
+  <si>
     <t>Amatsu</t>
   </si>
   <si>
-    <t>LAGO Gent Rozebroeken</t>
-  </si>
-  <si>
     <t>Firenze</t>
   </si>
   <si>
@@ -343,18 +346,36 @@
     <t>Prima Donna</t>
   </si>
   <si>
+    <t>Martino</t>
+  </si>
+  <si>
     <t>Brasserie Latem</t>
   </si>
   <si>
-    <t>Martino</t>
-  </si>
-  <si>
-    <t>La Dolce Vita</t>
-  </si>
-  <si>
     <t>Il Cortile 🇮🇹</t>
   </si>
   <si>
+    <t>'t Veer</t>
+  </si>
+  <si>
+    <t>Maximiliaan</t>
+  </si>
+  <si>
+    <t>Amadeus Gent 2 - Belfort</t>
+  </si>
+  <si>
+    <t>Tokyo Sushi Ghent</t>
+  </si>
+  <si>
+    <t>Jan van den Bon</t>
+  </si>
+  <si>
+    <t>'t Vosken</t>
+  </si>
+  <si>
+    <t>MULTATULI</t>
+  </si>
+  <si>
     <t>Friterie de l'Hôtel de Ville</t>
   </si>
   <si>
@@ -376,9 +397,18 @@
     <t>Bouillon De La Paix</t>
   </si>
   <si>
+    <t>ADANA</t>
+  </si>
+  <si>
     <t>Hameau de la Becque</t>
   </si>
   <si>
+    <t>KFC Lilles Lezennes</t>
+  </si>
+  <si>
+    <t>Estaminet Chez La Vieille</t>
+  </si>
+  <si>
     <t>La Fiesta</t>
   </si>
   <si>
@@ -391,34 +421,16 @@
     <t>La Ferme des Menhirs</t>
   </si>
   <si>
+    <t>Le Pavé Gourmand</t>
+  </si>
+  <si>
     <t>Yukito Sushi</t>
   </si>
   <si>
     <t>Le Soleil De Tunis</t>
   </si>
   <si>
-    <t>Pizzeria Chez Toni</t>
-  </si>
-  <si>
-    <t>Assiette au boeuf</t>
-  </si>
-  <si>
-    <t>Pizza Loossoise</t>
-  </si>
-  <si>
-    <t>Sushirama</t>
-  </si>
-  <si>
-    <t>Le Ch'ti Charivari</t>
-  </si>
-  <si>
-    <t>La Brasserie Jules</t>
-  </si>
-  <si>
-    <t>Les Orfèvres</t>
-  </si>
-  <si>
-    <t>Class'croute</t>
+    <t>La Bascule Du Petit Sancourt</t>
   </si>
   <si>
     <t>RESTAURANT LE STROMBOLI -RESTAURANT-PIZZÉRIA BAPAUME ET ENVIRONS</t>
@@ -427,49 +439,61 @@
     <t>Auberge de la Vallée d'Ancre</t>
   </si>
   <si>
-    <t>Sogeres</t>
-  </si>
-  <si>
-    <t>Restaurant Scolaire</t>
-  </si>
-  <si>
-    <t>Le Palais de Chine</t>
+    <t>Aux Gars du Nord</t>
+  </si>
+  <si>
+    <t>Le Méditerranée Sarl</t>
+  </si>
+  <si>
+    <t>Macdo</t>
+  </si>
+  <si>
+    <t>À la Chouette Gourmande</t>
+  </si>
+  <si>
+    <t>Rosiéres Kebab 80170</t>
+  </si>
+  <si>
+    <t>La Roselière</t>
   </si>
   <si>
     <t>Casa De Marco</t>
   </si>
   <si>
-    <t>Le Picardie</t>
-  </si>
-  <si>
-    <t>Restaurant Du Golf Club</t>
-  </si>
-  <si>
-    <t>Planet Asia</t>
-  </si>
-  <si>
-    <t>Le Verger D'Istanbul</t>
-  </si>
-  <si>
-    <t>Le Select</t>
-  </si>
-  <si>
-    <t>LIFI SOMME</t>
-  </si>
-  <si>
-    <t>Grill Istanbul</t>
-  </si>
-  <si>
-    <t>St Pierre Kebab</t>
-  </si>
-  <si>
-    <t>La vallée gourmande</t>
-  </si>
-  <si>
-    <t>Les Bouchons Damour</t>
-  </si>
-  <si>
-    <t>O'SWIFT Pizza</t>
+    <t>La Taverne du Cochon Salé</t>
+  </si>
+  <si>
+    <t>Le Bistrot D'Antoine</t>
+  </si>
+  <si>
+    <t>Le Comptoir de Marius</t>
+  </si>
+  <si>
+    <t>Le Saint Pierre</t>
+  </si>
+  <si>
+    <t>Asia Gourmet</t>
+  </si>
+  <si>
+    <t>Le Welcome</t>
+  </si>
+  <si>
+    <t>Le Chantilly</t>
+  </si>
+  <si>
+    <t>Pizza Délice</t>
+  </si>
+  <si>
+    <t>Stand Bienvillers Au Bois</t>
+  </si>
+  <si>
+    <t>SAS Som'baker</t>
+  </si>
+  <si>
+    <t>Hostellerie de la Croix d'Or</t>
+  </si>
+  <si>
+    <t>Pizza Anna</t>
   </si>
   <si>
     <t>Le Stromboli</t>
@@ -535,15 +559,9 @@
     <t>French Touch Compiègne</t>
   </si>
   <si>
-    <t>Huidenvettersplein 12, Brugge</t>
-  </si>
-  <si>
     <t>Beukenhofstraat 43, Anzegem</t>
   </si>
   <si>
-    <t>Vlamingstraat 5, Brugge</t>
-  </si>
-  <si>
     <t>Riemegemstraat 1, Kruisem</t>
   </si>
   <si>
@@ -553,15 +571,12 @@
     <t>Korenlei 2, Gent</t>
   </si>
   <si>
+    <t>Jakobijnenstraat 1, Gent</t>
+  </si>
+  <si>
     <t>Koningin Maria Hendrikaplein 65A, Gent</t>
   </si>
   <si>
-    <t>Jakobijnenstraat 1, Gent</t>
-  </si>
-  <si>
-    <t>Oostmeers 130, Brugge</t>
-  </si>
-  <si>
     <t>Urselweg 100, Maldegem</t>
   </si>
   <si>
@@ -571,12 +586,12 @@
     <t>Zuidstationstraat 14, Gent</t>
   </si>
   <si>
+    <t>Victor Braeckmanlaan 180/B, Gent</t>
+  </si>
+  <si>
     <t>Nederkouter 139, Gent</t>
   </si>
   <si>
-    <t>Victor Braeckmanlaan 180/B, Gent</t>
-  </si>
-  <si>
     <t>Sint-Amandstraat 1, Gent</t>
   </si>
   <si>
@@ -586,18 +601,36 @@
     <t>Overpoortstraat 46, Gent</t>
   </si>
   <si>
+    <t>Vlaanderenstraat 125, Gent</t>
+  </si>
+  <si>
     <t>Kortrijksesteenweg 9, Sint-Martens-Latem</t>
   </si>
   <si>
-    <t>Vlaanderenstraat 125, Gent</t>
-  </si>
-  <si>
-    <t>Stationsstraat 10, Kortrijk</t>
-  </si>
-  <si>
     <t>Kraanlei 53, Gent</t>
   </si>
   <si>
+    <t>Berchemweg 191, Oudenaarde</t>
+  </si>
+  <si>
+    <t>Mageleinstraat 50, Gent</t>
+  </si>
+  <si>
+    <t>Goudenleeuwplein 7, Gent</t>
+  </si>
+  <si>
+    <t>Botermarkt 10, Gent</t>
+  </si>
+  <si>
+    <t>Floraliënlaan 22, Gent</t>
+  </si>
+  <si>
+    <t>Sint-Baafsplein 19, Gent</t>
+  </si>
+  <si>
+    <t>Huidevetterskaai 40, Gent</t>
+  </si>
+  <si>
     <t>Place Van Gogh, Villeneuve-d'Ascq</t>
   </si>
   <si>
@@ -619,9 +652,18 @@
     <t>25 Place Rihour, Lille</t>
   </si>
   <si>
+    <t>Rue Dorez 15, Tournai</t>
+  </si>
+  <si>
     <t>14 Rue de la Becque, Avelin</t>
   </si>
   <si>
+    <t>Rue de Chanzy - Lezennes, Lezennes</t>
+  </si>
+  <si>
+    <t>60 Rue de Gand, Lille</t>
+  </si>
+  <si>
     <t>102 Boulevard Emile Basly, Lens</t>
   </si>
   <si>
@@ -634,34 +676,16 @@
     <t>Rue de la Fraternité, Acq</t>
   </si>
   <si>
+    <t>113 Rue Léon Rudent, Orchies</t>
+  </si>
+  <si>
     <t>33 Rue de Paris, Douai</t>
   </si>
   <si>
     <t>24 Rue Merlin de Douai, Douai</t>
   </si>
   <si>
-    <t>44 Rue Cyprien Quinet, Carvin</t>
-  </si>
-  <si>
-    <t>56 Grand'Place, Arras</t>
-  </si>
-  <si>
-    <t>10 Place de la République, Loos-en-Gohelle</t>
-  </si>
-  <si>
-    <t>14 Rue Saint-Patrice, Amiens</t>
-  </si>
-  <si>
-    <t>52 Rue des Jacobins, Amiens</t>
-  </si>
-  <si>
-    <t>18 Boulevard d'Alsace Lorraine, Amiens</t>
-  </si>
-  <si>
-    <t>14 Rue des Orfèvres, Amiens</t>
-  </si>
-  <si>
-    <t>56 Rue des Jacobins, Amiens</t>
+    <t>80 Route nationale 43, Sancourt</t>
   </si>
   <si>
     <t>37 Faubourg de Péronne, Bapaume</t>
@@ -670,49 +694,61 @@
     <t>6 Rue du Moulin, Authuille</t>
   </si>
   <si>
-    <t>Rue Titien, Amiens</t>
-  </si>
-  <si>
-    <t>18 Rue des Déportés, Camon</t>
-  </si>
-  <si>
-    <t>174 Avenue Henri Barbusse, Longueau</t>
+    <t>30 Rue Saint-Sauveur, Péronne</t>
+  </si>
+  <si>
+    <t>21 Rue Béranger, Péronne</t>
+  </si>
+  <si>
+    <t>Lille, A1, Péronne</t>
+  </si>
+  <si>
+    <t>25 Route de Paris, Péronne</t>
+  </si>
+  <si>
+    <t>13 Rue du Maréchal Foch, Rosières-en-Santerre</t>
+  </si>
+  <si>
+    <t>7 Rue Jean Jaurès, Roisel</t>
   </si>
   <si>
     <t>3 Rue Aristide Briand, Fouilloy</t>
   </si>
   <si>
-    <t>Port d'Amont, Amiens</t>
-  </si>
-  <si>
-    <t>RD929, Querrieu</t>
-  </si>
-  <si>
-    <t>3 Avenue de l'Arc, Longueau</t>
-  </si>
-  <si>
-    <t>50 Rue de la Vigne, Flesselles</t>
-  </si>
-  <si>
-    <t>2ter Rue Louis Prot, Longueau</t>
-  </si>
-  <si>
-    <t>47 Place René Goblet, Amiens</t>
-  </si>
-  <si>
-    <t>1 Boulevard de Bapaume, Amiens</t>
-  </si>
-  <si>
-    <t>119 Chaussée Saint-Pierre, Amiens</t>
-  </si>
-  <si>
-    <t>23 Rue de la Vallée, Amiens</t>
-  </si>
-  <si>
-    <t>50 Rue du Vivier, Amiens</t>
-  </si>
-  <si>
-    <t>37 Rue Jules Barni, Amiens</t>
+    <t>29 Rue d'Albert, Authuille</t>
+  </si>
+  <si>
+    <t>8 Place André Audinot, Péronne</t>
+  </si>
+  <si>
+    <t>Route de Rosières, Roye</t>
+  </si>
+  <si>
+    <t>3 Rue Delambre, Lamotte-Warfusée</t>
+  </si>
+  <si>
+    <t>ZONE EMILE PLUCHET, Route de Rosières, Roye</t>
+  </si>
+  <si>
+    <t>12 Avenue du Général de Gaulle, Roye</t>
+  </si>
+  <si>
+    <t>10B Rue de Saint-Léger, Croisilles</t>
+  </si>
+  <si>
+    <t>14 Rue du Docteur Duquesnel, Roye</t>
+  </si>
+  <si>
+    <t>d'Hannescamps,, Le Chemin d'Hannescamps, Bienvillers-au-Bois</t>
+  </si>
+  <si>
+    <t>26 B Route nationale, Rancourt</t>
+  </si>
+  <si>
+    <t>123 Rue Saint-Gilles, Roye</t>
+  </si>
+  <si>
+    <t>45 Rue du Général Leclerc, Ham</t>
   </si>
   <si>
     <t>Accès, 12 Rue des Cordeliers, 2 Rue des Lombards, Compiègne</t>
@@ -781,21 +817,15 @@
     <t>restaurant, food, point_of_interest, establishment</t>
   </si>
   <si>
+    <t>restaurant, health, food, point_of_interest, establishment</t>
+  </si>
+  <si>
     <t>restaurant, point_of_interest, food, establishment</t>
   </si>
   <si>
-    <t>health, restaurant, food, point_of_interest, establishment</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.2077243,3.227483099999999&amp;query_place_id=ChIJkaD3fMVQw0cR0Y-SgHCHlvw</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.8354964,3.3953747&amp;query_place_id=ChIJv8_dynU9w0cRPwuu4Hw6BCM</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.2095128,3.2245342&amp;query_place_id=ChIJD_pZGNBQw0cRD-WANdpmDGk</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.9036673,3.5096569&amp;query_place_id=ChIJ6U6ntWgUw0cRZrq8q_ohqUU</t>
   </si>
   <si>
@@ -805,15 +835,12 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.05561119999999,3.7205134&amp;query_place_id=ChIJd92M2UBxw0cRcLC_XWtAw5M</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0521389,3.7201179&amp;query_place_id=ChIJcw76AERxw0cRCZ9UPLL7szA</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0372949,3.7103165&amp;query_place_id=ChIJfXFDIWBxw0cRE9YYAtd17F4</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0521389,3.7201179&amp;query_place_id=ChIJcw76AERxw0cRCZ9UPLL7szA</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.1998871,3.220129899999999&amp;query_place_id=ChIJO6D6ut1Qw0cRfRITh057Upg</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.16801830000001,3.4724922&amp;query_place_id=ChIJYdFddZ1nw0cRf0zN9IQqQ7Q</t>
   </si>
   <si>
@@ -823,12 +850,12 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0490043,3.732778999999999&amp;query_place_id=ChIJ66An1k1xw0cRrkKcb_6Z488</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0595473,3.761043&amp;query_place_id=ChIJl4CsVsF2w0cRytpeXShIbNE</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0465092,3.7225456&amp;query_place_id=ChIJI46pG0dxw0cRIXbgTe31oZc</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0595473,3.761043&amp;query_place_id=ChIJl4CsVsF2w0cRytpeXShIbNE</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0438889,3.7247222&amp;query_place_id=ChIJvwaiZ1pxw0cRITmiV6KwtPw</t>
   </si>
   <si>
@@ -838,18 +865,36 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0403269,3.725390500000001&amp;query_place_id=ChIJZ6VMYFdxw0cRfVoCvTscwOg</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.04891989999999,3.7312643&amp;query_place_id=ChIJl8_4Z05xw0cRY8fapfMJrxc</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0140263,3.6491051&amp;query_place_id=ChIJr82_7G1yw0cRebseGTV57d0</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.04891989999999,3.7312643&amp;query_place_id=ChIJl8_4Z05xw0cRY8fapfMJrxc</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.8255556,3.2641667&amp;query_place_id=ChIJocMKhOE6w0cRiwy8ypm_OLY</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.05728250000001,3.7231798&amp;query_place_id=ChIJD8S0YEdxw0cRfVs16dksyJQ</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.81935849999999,3.5751952&amp;query_place_id=ChIJi-zbr0UQw0cRyBDtc11VPiE</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.052705,3.724562499999999&amp;query_place_id=ChIJyXZkekZxw0cRb9uqej8bxZY</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.05421639999999,3.7240936&amp;query_place_id=ChIJs0g1-kZxw0cR46lPwxTdOpg</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0540422,3.7255715&amp;query_place_id=ChIJU1sJSUZxw0cRgmHC8o3MZwQ</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.03981009999999,3.718738&amp;query_place_id=ChIJ0X-9015xw0cRsPLuG79Kn4s</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.05352310000001,3.726121400000001&amp;query_place_id=ChIJO5B6a0Zxw0cRCSaWrQEL7bE</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=51.061058,3.72782&amp;query_place_id=ChIJW3OtxDlxw0cRM_nXQaujiBg</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.61939779999999,3.132437599999999&amp;query_place_id=ChIJmzeJyjnWwkcRCMoN538F2as</t>
   </si>
   <si>
@@ -871,9 +916,18 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.63577600000001,3.0634036&amp;query_place_id=ChIJCQOYnYjVwkcR6lYaR-xTg98</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.606813,3.382719799999999&amp;query_place_id=ChIJn9OLi97fwkcRN9zVioh1KUc</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.5243349,3.0756846&amp;query_place_id=ChIJGV-_vdfTwkcRX88cSrHGyf8</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.61273699999999,3.123373&amp;query_place_id=ChIJiXvXemrWwkcR1Th5LFqOW7s</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.6427316,3.0668892&amp;query_place_id=ChIJb-2V4XYqw0cRcdf1yjoy0F8</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.43022910000001,2.8241761&amp;query_place_id=ChIJbx9ih_Aw3UcRoGOf2o5HMr4</t>
   </si>
   <si>
@@ -886,34 +940,16 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.3472046,2.6535711&amp;query_place_id=ChIJ1WAX4MM-3UcRMMlIwokR7OY</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.4796752,3.237034299999999&amp;query_place_id=ChIJPdx5aSXbwkcRQhNCE1K7LD4</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.367342,3.081729999999999&amp;query_place_id=ChIJ3d3K12fJwkcR0dksDPOE-LE</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.3691968,3.078329&amp;query_place_id=ChIJI5GNfGfJwkcRkvhp-n7tsQo</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.4912933,2.9707772&amp;query_place_id=ChIJe_MMnkYt3UcRc-auwbiNW0c</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.2920298,2.7812821&amp;query_place_id=ChIJ-V0ngnRI3UcRxNYJAxiXTqM</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.457384,2.793196&amp;query_place_id=ChIJV7YKDXUw3UcRFedUAMyku0M</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.895006,2.296499&amp;query_place_id=ChIJs-JfFD-E50cRkks1dAfeD04</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8912279,2.3000171&amp;query_place_id=ChIJod-1BEeE50cRGEbTCldDiEk</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.89197739999999,2.3079003&amp;query_place_id=ChIJKTehx0mE50cRRBnfjWRP2e8</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8958208,2.2991908&amp;query_place_id=ChIJGTko2DiE50cRmeo-Et037Rs</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8908424,2.300658200000001&amp;query_place_id=ChIJT7GmqkeE50cRjqo3SaXmEFs</t>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.2091985,3.1905208&amp;query_place_id=ChIJMdnRjTG6wkcRhoM1KoA2Xl8</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.0990133,2.8551931&amp;query_place_id=ChIJdU5gH9dT3UcRL5zDVej010Y</t>
@@ -922,49 +958,61 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.0440674,2.666995500000001&amp;query_place_id=ChIJ2WXVuTBZ3UcRf0B-9mmdb1Q</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.92263819999999,2.2929843&amp;query_place_id=ChIJ-W2FEpiG50cRVoTEf_6176I</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.89451709999999,2.3414744&amp;query_place_id=ChIJY2VhcpGF50cRSy6NwjYOsPo</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.868616,2.3609755&amp;query_place_id=ChIJsRkGiICP50cR4y6APgUdWNA</t>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.9306446,2.9373479&amp;query_place_id=ChIJz9Z6O4UA6EcRRbZGn3G3gbM</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.9294497,2.9385445&amp;query_place_id=ChIJaYuwuJoA6EcRk7-jwtLVO8g</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.887574,2.837822&amp;query_place_id=ChIJtTuE06D-50cR2--b95hIc8I</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.9157805,2.9340714&amp;query_place_id=ChIJib4_kqMA6EcRD6sUNY4aftQ</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.812285,2.7008719&amp;query_place_id=ChIJaaZMOMPv50cRV7HwbArC9bQ</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.9470246,3.1002615&amp;query_place_id=ChIJ81iJTsMC6EcRB7QQZNBe63c</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.9000698,2.5028801&amp;query_place_id=ChIJu9TW-YeM50cRWgv1BJZBEA0</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.89527159999999,2.307976500000001&amp;query_place_id=ChIJT-FpWzaE50cR1O3LCiccUps</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.9243809,2.3902492&amp;query_place_id=ChIJ866YABOJ50cR64ETj_MHZBM</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8690513,2.3706788&amp;query_place_id=ChIJG910IIOP50cRXrfJdLILZ2Y</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.00485090000001,2.2640913&amp;query_place_id=ChIJvb4H_Rp-3UcR3lsWBx04w6U</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.87036320000001,2.3566902&amp;query_place_id=ChIJQcUaDH-F50cRis_9pkrt7CY</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8912963,2.3038483&amp;query_place_id=ChIJ4SFseEiE50cReLJiUM2S_o8</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8821619,2.3188738&amp;query_place_id=ChIJmTVfja2F50cRk-m6tyEg5ic</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.9033033,2.3055391&amp;query_place_id=ChIJhwejHDCE50cRyPI1ZjgtwAU</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8918596,2.309983700000001&amp;query_place_id=ChIJ8fgtIkqE50cRhFjeGhOUc-k</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8924005,2.308677899999999&amp;query_place_id=ChIJRfSU7kmE50cRZUAzMfzB-CU</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.88939339999999,2.3103845&amp;query_place_id=ChIJcYYKwkuE50cRM00saJuEInU</t>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.0409911,2.6686785&amp;query_place_id=ChIJxxW9nDpZ3UcRq2W4vQBjXdo</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.9291968,2.933116499999999&amp;query_place_id=ChIJqbcdlZwA6EcRwvpe_YOrcIA</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.7097598,2.773197300000001&amp;query_place_id=ChIJ1QnuayDn50cR2Dz4I-QJwz8</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.8708087,2.5975248&amp;query_place_id=ChIJl5YJwavz50cRrswjHSVYqX4</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.7089958,2.773895500000001&amp;query_place_id=ChIJA-D9f_rm50cR3alW2glvv0s</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.6995639,2.7944886&amp;query_place_id=ChIJO4XZwNjm50cR7TkMIfUH8i0</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.1980106,2.8759627&amp;query_place_id=ChIJf6fIWTBM3UcR481vvWP5QAk</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.6978505,2.791623399999999&amp;query_place_id=ChIJ0b2ioiDn50cRSacFMQFo1gs</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.17135099999999,2.6318673&amp;query_place_id=ChIJx0IhISND3UcRulMyFL2o8-A</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=50.0034562,2.911265&amp;query_place_id=ChIJZ5IoFBVV3UcRfzObqtmTFuw</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.6905687,2.788442&amp;query_place_id=ChIJEQnn8yLn50cRGCqPPfadcEk</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=49.7447927,3.0752862&amp;query_place_id=ChIJVToX4xIO6EcRcQvXHvdfhpA</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.41652569999999,2.8255822&amp;query_place_id=ChIJ3fl0IYHW50cR_mvDeqFjsfs</t>
@@ -1398,7 +1446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -1441,34 +1489,34 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="D2">
-        <v>51.2077243</v>
+        <v>50.8354964</v>
       </c>
       <c r="E2">
-        <v>3.227483099999999</v>
+        <v>3.3953747</v>
       </c>
       <c r="F2">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="G2">
-        <v>1727</v>
+        <v>247</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1476,34 +1524,34 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D3">
-        <v>50.8354964</v>
+        <v>50.9036673</v>
       </c>
       <c r="E3">
-        <v>3.3953747</v>
+        <v>3.5096569</v>
       </c>
       <c r="F3">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="G3">
-        <v>246</v>
+        <v>728</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I3" t="b">
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1511,22 +1559,22 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D4">
-        <v>51.2095128</v>
+        <v>51.0551243</v>
       </c>
       <c r="E4">
-        <v>3.2245342</v>
+        <v>3.721278300000001</v>
       </c>
       <c r="F4">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="G4">
-        <v>396</v>
+        <v>1552</v>
       </c>
       <c r="H4">
         <v>2</v>
@@ -1535,10 +1583,10 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1546,34 +1594,34 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="D5">
-        <v>50.9036673</v>
+        <v>51.05561119999999</v>
       </c>
       <c r="E5">
-        <v>3.5096569</v>
+        <v>3.7205134</v>
       </c>
       <c r="F5">
-        <v>4.7</v>
+        <v>3.8</v>
       </c>
       <c r="G5">
-        <v>728</v>
+        <v>525</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1581,22 +1629,22 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D6">
-        <v>51.0551243</v>
+        <v>51.0521389</v>
       </c>
       <c r="E6">
-        <v>3.721278300000001</v>
+        <v>3.7201179</v>
       </c>
       <c r="F6">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>1551</v>
+        <v>1311</v>
       </c>
       <c r="H6">
         <v>2</v>
@@ -1605,10 +1653,10 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1616,34 +1664,34 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="D7">
-        <v>51.05561119999999</v>
+        <v>51.0372949</v>
       </c>
       <c r="E7">
-        <v>3.7205134</v>
+        <v>3.7103165</v>
       </c>
       <c r="F7">
-        <v>3.8</v>
+        <v>4.3</v>
       </c>
       <c r="G7">
-        <v>525</v>
+        <v>683</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1651,34 +1699,34 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D8">
-        <v>51.0372949</v>
+        <v>51.16801830000001</v>
       </c>
       <c r="E8">
-        <v>3.7103165</v>
+        <v>3.4724922</v>
       </c>
       <c r="F8">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="G8">
-        <v>683</v>
+        <v>757</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1686,22 +1734,22 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="D9">
-        <v>51.0521389</v>
+        <v>51.0567995</v>
       </c>
       <c r="E9">
-        <v>3.7201179</v>
+        <v>3.7196267</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="G9">
-        <v>1310</v>
+        <v>2128</v>
       </c>
       <c r="H9">
         <v>2</v>
@@ -1710,10 +1758,10 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1721,22 +1769,22 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="D10">
-        <v>51.1998871</v>
+        <v>51.0490043</v>
       </c>
       <c r="E10">
-        <v>3.220129899999999</v>
+        <v>3.732778999999999</v>
       </c>
       <c r="F10">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="G10">
-        <v>794</v>
+        <v>352</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -1745,10 +1793,10 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1756,34 +1804,31 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D11">
-        <v>51.16801830000001</v>
+        <v>51.0595473</v>
       </c>
       <c r="E11">
-        <v>3.4724922</v>
+        <v>3.761043</v>
       </c>
       <c r="F11">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>756</v>
-      </c>
-      <c r="H11">
-        <v>2</v>
+        <v>6396</v>
       </c>
       <c r="I11" t="b">
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1791,34 +1836,34 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D12">
-        <v>51.0567995</v>
+        <v>51.0465092</v>
       </c>
       <c r="E12">
-        <v>3.7196267</v>
+        <v>3.7225456</v>
       </c>
       <c r="F12">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="G12">
-        <v>2128</v>
+        <v>386</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1826,34 +1871,34 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="D13">
-        <v>51.0490043</v>
+        <v>51.0438889</v>
       </c>
       <c r="E13">
-        <v>3.732778999999999</v>
+        <v>3.7247222</v>
       </c>
       <c r="F13">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G13">
-        <v>352</v>
+        <v>1103</v>
       </c>
       <c r="H13">
         <v>2</v>
       </c>
       <c r="I13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1861,34 +1906,34 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="D14">
-        <v>51.0465092</v>
+        <v>51.0522725</v>
       </c>
       <c r="E14">
-        <v>3.7225456</v>
+        <v>3.7198882</v>
       </c>
       <c r="F14">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="G14">
-        <v>386</v>
+        <v>348</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I14" t="b">
         <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1896,31 +1941,34 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="D15">
-        <v>51.0595473</v>
+        <v>51.0403269</v>
       </c>
       <c r="E15">
-        <v>3.761043</v>
+        <v>3.725390500000001</v>
       </c>
       <c r="F15">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="G15">
-        <v>6396</v>
+        <v>728</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
       </c>
       <c r="I15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1928,34 +1976,34 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="D16">
-        <v>51.0438889</v>
+        <v>51.04891989999999</v>
       </c>
       <c r="E16">
-        <v>3.7247222</v>
+        <v>3.7312643</v>
       </c>
       <c r="F16">
         <v>4.5</v>
       </c>
       <c r="G16">
-        <v>1102</v>
+        <v>308</v>
       </c>
       <c r="H16">
         <v>2</v>
       </c>
       <c r="I16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1963,34 +2011,34 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="D17">
-        <v>51.0522725</v>
+        <v>51.0140263</v>
       </c>
       <c r="E17">
-        <v>3.7198882</v>
+        <v>3.6491051</v>
       </c>
       <c r="F17">
-        <v>4.1</v>
+        <v>4.4</v>
       </c>
       <c r="G17">
-        <v>348</v>
+        <v>412</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1998,34 +2046,34 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C18" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="D18">
-        <v>51.0403269</v>
+        <v>51.05728250000001</v>
       </c>
       <c r="E18">
-        <v>3.725390500000001</v>
+        <v>3.7231798</v>
       </c>
       <c r="F18">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="G18">
-        <v>727</v>
+        <v>829</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2033,34 +2081,34 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D19">
-        <v>51.0140263</v>
+        <v>50.81935849999999</v>
       </c>
       <c r="E19">
-        <v>3.6491051</v>
+        <v>3.5751952</v>
       </c>
       <c r="F19">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="G19">
-        <v>412</v>
+        <v>924</v>
       </c>
       <c r="H19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2068,22 +2116,22 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C20" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="D20">
-        <v>51.04891989999999</v>
+        <v>51.052705</v>
       </c>
       <c r="E20">
-        <v>3.7312643</v>
+        <v>3.724562499999999</v>
       </c>
       <c r="F20">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="G20">
-        <v>307</v>
+        <v>870</v>
       </c>
       <c r="H20">
         <v>2</v>
@@ -2092,10 +2140,10 @@
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2103,34 +2151,34 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="D21">
-        <v>50.8255556</v>
+        <v>51.05421639999999</v>
       </c>
       <c r="E21">
-        <v>3.2641667</v>
+        <v>3.7240936</v>
       </c>
       <c r="F21">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="G21">
-        <v>467</v>
+        <v>3834</v>
       </c>
       <c r="H21">
         <v>2</v>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2138,34 +2186,34 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C22" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D22">
-        <v>51.05728250000001</v>
+        <v>51.0540422</v>
       </c>
       <c r="E22">
-        <v>3.7231798</v>
+        <v>3.7255715</v>
       </c>
       <c r="F22">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="G22">
-        <v>829</v>
+        <v>805</v>
       </c>
       <c r="H22">
         <v>2</v>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2173,31 +2221,31 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C23" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="D23">
-        <v>50.61939779999999</v>
+        <v>51.03981009999999</v>
       </c>
       <c r="E23">
-        <v>3.132437599999999</v>
+        <v>3.718738</v>
       </c>
       <c r="F23">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="G23">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="I23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2205,34 +2253,34 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C24" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="D24">
-        <v>50.8500201</v>
+        <v>51.05352310000001</v>
       </c>
       <c r="E24">
-        <v>2.881268900000001</v>
+        <v>3.726121400000001</v>
       </c>
       <c r="F24">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="G24">
-        <v>609</v>
+        <v>2022</v>
       </c>
       <c r="H24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2240,31 +2288,34 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="D25">
-        <v>50.78213179999999</v>
+        <v>51.061058</v>
       </c>
       <c r="E25">
-        <v>3.0023986</v>
+        <v>3.72782</v>
       </c>
       <c r="F25">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="G25">
-        <v>3498</v>
+        <v>1351</v>
+      </c>
+      <c r="H25">
+        <v>2</v>
       </c>
       <c r="I25" t="b">
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -2272,34 +2323,31 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="D26">
-        <v>50.64078540000001</v>
+        <v>50.61939779999999</v>
       </c>
       <c r="E26">
-        <v>3.061416099999999</v>
+        <v>3.132437599999999</v>
       </c>
       <c r="F26">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="G26">
-        <v>519</v>
-      </c>
-      <c r="H26">
-        <v>2</v>
+        <v>127</v>
       </c>
       <c r="I26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2307,34 +2355,34 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C27" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="D27">
-        <v>50.8263743</v>
+        <v>50.8500201</v>
       </c>
       <c r="E27">
-        <v>3.1773917</v>
+        <v>2.881268900000001</v>
       </c>
       <c r="F27">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G27">
-        <v>660</v>
+        <v>610</v>
       </c>
       <c r="H27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2342,34 +2390,31 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C28" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D28">
-        <v>50.7344444</v>
+        <v>50.78213179999999</v>
       </c>
       <c r="E28">
-        <v>3.2863889</v>
+        <v>3.0023986</v>
       </c>
       <c r="F28">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="G28">
-        <v>2984</v>
-      </c>
-      <c r="H28">
-        <v>2</v>
+        <v>3498</v>
       </c>
       <c r="I28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2377,34 +2422,34 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C29" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="D29">
-        <v>50.63577600000001</v>
+        <v>50.64078540000001</v>
       </c>
       <c r="E29">
-        <v>3.0634036</v>
+        <v>3.061416099999999</v>
       </c>
       <c r="F29">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="G29">
-        <v>1199</v>
+        <v>519</v>
       </c>
       <c r="H29">
         <v>2</v>
       </c>
       <c r="I29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2412,31 +2457,34 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="D30">
-        <v>50.5243349</v>
+        <v>50.8263743</v>
       </c>
       <c r="E30">
-        <v>3.0756846</v>
+        <v>3.1773917</v>
       </c>
       <c r="F30">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="G30">
-        <v>124</v>
+        <v>660</v>
+      </c>
+      <c r="H30">
+        <v>2</v>
       </c>
       <c r="I30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2444,31 +2492,34 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C31" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="D31">
-        <v>50.43022910000001</v>
+        <v>50.7344444</v>
       </c>
       <c r="E31">
-        <v>2.8241761</v>
+        <v>3.2863889</v>
       </c>
       <c r="F31">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="G31">
-        <v>429</v>
+        <v>2984</v>
+      </c>
+      <c r="H31">
+        <v>2</v>
       </c>
       <c r="I31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2476,34 +2527,34 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C32" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="D32">
-        <v>50.42831</v>
+        <v>50.63577600000001</v>
       </c>
       <c r="E32">
-        <v>2.826468599999999</v>
+        <v>3.0634036</v>
       </c>
       <c r="F32">
-        <v>4.1</v>
+        <v>3.8</v>
       </c>
       <c r="G32">
-        <v>847</v>
+        <v>1199</v>
       </c>
       <c r="H32">
         <v>2</v>
       </c>
       <c r="I32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2511,34 +2562,34 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C33" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="D33">
-        <v>50.2927725</v>
+        <v>50.606813</v>
       </c>
       <c r="E33">
-        <v>2.780148199999999</v>
+        <v>3.382719799999999</v>
       </c>
       <c r="F33">
         <v>4.3</v>
       </c>
       <c r="G33">
-        <v>690</v>
+        <v>598</v>
       </c>
       <c r="H33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2546,28 +2597,31 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" t="s">
+        <v>213</v>
+      </c>
+      <c r="D34">
+        <v>50.5243349</v>
+      </c>
+      <c r="E34">
+        <v>3.0756846</v>
+      </c>
+      <c r="F34">
+        <v>4.4</v>
+      </c>
+      <c r="G34">
         <v>124</v>
       </c>
-      <c r="C34" t="s">
-        <v>205</v>
-      </c>
-      <c r="D34">
-        <v>50.3472046</v>
-      </c>
-      <c r="E34">
-        <v>2.6535711</v>
-      </c>
-      <c r="F34">
-        <v>4.8</v>
-      </c>
-      <c r="G34">
-        <v>163</v>
+      <c r="I34" t="b">
+        <v>0</v>
       </c>
       <c r="J34" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2575,34 +2629,34 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C35" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="D35">
-        <v>50.367342</v>
+        <v>50.61273699999999</v>
       </c>
       <c r="E35">
-        <v>3.081729999999999</v>
+        <v>3.123373</v>
       </c>
       <c r="F35">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="G35">
-        <v>376</v>
+        <v>4178</v>
       </c>
       <c r="H35">
         <v>2</v>
       </c>
       <c r="I35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2610,34 +2664,34 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C36" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="D36">
-        <v>50.3691968</v>
+        <v>50.6427316</v>
       </c>
       <c r="E36">
-        <v>3.078329</v>
+        <v>3.0668892</v>
       </c>
       <c r="F36">
         <v>4.5</v>
       </c>
       <c r="G36">
-        <v>464</v>
+        <v>4716</v>
       </c>
       <c r="H36">
         <v>2</v>
       </c>
       <c r="I36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2645,34 +2699,31 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="D37">
-        <v>50.4912933</v>
+        <v>50.43022910000001</v>
       </c>
       <c r="E37">
-        <v>2.9707772</v>
+        <v>2.8241761</v>
       </c>
       <c r="F37">
-        <v>4.1</v>
+        <v>4.6</v>
       </c>
       <c r="G37">
-        <v>52</v>
-      </c>
-      <c r="H37">
-        <v>2</v>
+        <v>429</v>
       </c>
       <c r="I37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2680,34 +2731,34 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C38" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="D38">
-        <v>50.2920298</v>
+        <v>50.42831</v>
       </c>
       <c r="E38">
-        <v>2.7812821</v>
+        <v>2.826468599999999</v>
       </c>
       <c r="F38">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="G38">
-        <v>2541</v>
+        <v>847</v>
       </c>
       <c r="H38">
         <v>2</v>
       </c>
       <c r="I38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2715,34 +2766,34 @@
         <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D39">
-        <v>50.457384</v>
+        <v>50.2927725</v>
       </c>
       <c r="E39">
-        <v>2.793196</v>
+        <v>2.780148199999999</v>
       </c>
       <c r="F39">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="G39">
-        <v>196</v>
+        <v>690</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2750,34 +2801,28 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="D40">
-        <v>49.895006</v>
+        <v>50.3472046</v>
       </c>
       <c r="E40">
-        <v>2.296499</v>
+        <v>2.6535711</v>
       </c>
       <c r="F40">
-        <v>4.1</v>
+        <v>4.8</v>
       </c>
       <c r="G40">
-        <v>1330</v>
-      </c>
-      <c r="H40">
-        <v>2</v>
-      </c>
-      <c r="I40" t="b">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="J40" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2785,34 +2830,34 @@
         <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C41" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="D41">
-        <v>49.8912279</v>
+        <v>50.4796752</v>
       </c>
       <c r="E41">
-        <v>2.3000171</v>
+        <v>3.237034299999999</v>
       </c>
       <c r="F41">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="G41">
-        <v>613</v>
+        <v>473</v>
       </c>
       <c r="H41">
         <v>2</v>
       </c>
       <c r="I41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2820,34 +2865,34 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C42" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D42">
-        <v>49.89197739999999</v>
+        <v>50.367342</v>
       </c>
       <c r="E42">
-        <v>2.3079003</v>
+        <v>3.081729999999999</v>
       </c>
       <c r="F42">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="G42">
-        <v>1697</v>
+        <v>376</v>
       </c>
       <c r="H42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2855,34 +2900,34 @@
         <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C43" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="D43">
-        <v>49.8958208</v>
+        <v>50.3691968</v>
       </c>
       <c r="E43">
-        <v>2.2991908</v>
+        <v>3.078329</v>
       </c>
       <c r="F43">
         <v>4.5</v>
       </c>
       <c r="G43">
-        <v>578</v>
+        <v>464</v>
       </c>
       <c r="H43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2890,34 +2935,34 @@
         <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C44" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="D44">
-        <v>49.8908424</v>
+        <v>50.2091985</v>
       </c>
       <c r="E44">
-        <v>2.300658200000001</v>
+        <v>3.1905208</v>
       </c>
       <c r="F44">
-        <v>4.1</v>
+        <v>3.8</v>
       </c>
       <c r="G44">
-        <v>94</v>
+        <v>398</v>
       </c>
       <c r="H44">
         <v>2</v>
       </c>
       <c r="I44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2925,10 +2970,10 @@
         <v>54</v>
       </c>
       <c r="B45" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C45" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D45">
         <v>50.0990133</v>
@@ -2946,13 +2991,13 @@
         <v>2</v>
       </c>
       <c r="I45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -2960,10 +3005,10 @@
         <v>55</v>
       </c>
       <c r="B46" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C46" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="D46">
         <v>50.0440674</v>
@@ -2981,13 +3026,13 @@
         <v>2</v>
       </c>
       <c r="I46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -2995,31 +3040,34 @@
         <v>56</v>
       </c>
       <c r="B47" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C47" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="D47">
-        <v>49.92263819999999</v>
+        <v>49.9306446</v>
       </c>
       <c r="E47">
-        <v>2.2929843</v>
+        <v>2.9373479</v>
       </c>
       <c r="F47">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="G47">
-        <v>25</v>
+        <v>687</v>
       </c>
       <c r="H47">
+        <v>2</v>
+      </c>
+      <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -3027,31 +3075,34 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C48" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="D48">
-        <v>49.89451709999999</v>
+        <v>49.9294497</v>
       </c>
       <c r="E48">
-        <v>2.3414744</v>
+        <v>2.9385445</v>
       </c>
       <c r="F48">
         <v>4.7</v>
       </c>
       <c r="G48">
-        <v>6</v>
+        <v>340</v>
+      </c>
+      <c r="H48">
+        <v>2</v>
       </c>
       <c r="I48" t="b">
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -3059,34 +3110,31 @@
         <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C49" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="D49">
-        <v>49.868616</v>
+        <v>49.887574</v>
       </c>
       <c r="E49">
-        <v>2.3609755</v>
+        <v>2.837822</v>
       </c>
       <c r="F49">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="G49">
-        <v>783</v>
-      </c>
-      <c r="H49">
-        <v>2</v>
+        <v>627</v>
       </c>
       <c r="I49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3094,34 +3142,31 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C50" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D50">
-        <v>49.9000698</v>
+        <v>49.9157805</v>
       </c>
       <c r="E50">
-        <v>2.5028801</v>
+        <v>2.9340714</v>
       </c>
       <c r="F50">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="G50">
-        <v>223</v>
-      </c>
-      <c r="H50">
-        <v>2</v>
+        <v>138</v>
       </c>
       <c r="I50" t="b">
         <v>0</v>
       </c>
       <c r="J50" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3129,31 +3174,34 @@
         <v>60</v>
       </c>
       <c r="B51" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C51" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D51">
-        <v>49.89527159999999</v>
+        <v>49.812285</v>
       </c>
       <c r="E51">
-        <v>2.307976500000001</v>
+        <v>2.7008719</v>
       </c>
       <c r="F51">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="G51">
-        <v>343</v>
+        <v>90</v>
+      </c>
+      <c r="H51">
+        <v>1</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3161,22 +3209,22 @@
         <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C52" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="D52">
-        <v>49.9243809</v>
+        <v>49.9470246</v>
       </c>
       <c r="E52">
-        <v>2.3902492</v>
+        <v>3.1002615</v>
       </c>
       <c r="F52">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="G52">
-        <v>227</v>
+        <v>183</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -3185,10 +3233,10 @@
         <v>0</v>
       </c>
       <c r="J52" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -3196,34 +3244,34 @@
         <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C53" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="D53">
-        <v>49.8690513</v>
+        <v>49.9000698</v>
       </c>
       <c r="E53">
-        <v>2.3706788</v>
+        <v>2.5028801</v>
       </c>
       <c r="F53">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="G53">
-        <v>2892</v>
+        <v>223</v>
       </c>
       <c r="H53">
         <v>2</v>
       </c>
       <c r="I53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -3231,34 +3279,34 @@
         <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C54" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D54">
-        <v>50.00485090000001</v>
+        <v>50.0409911</v>
       </c>
       <c r="E54">
-        <v>2.2640913</v>
+        <v>2.6686785</v>
       </c>
       <c r="F54">
         <v>4.6</v>
       </c>
       <c r="G54">
-        <v>421</v>
+        <v>581</v>
       </c>
       <c r="H54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -3266,34 +3314,34 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C55" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="D55">
-        <v>49.87036320000001</v>
+        <v>49.9291968</v>
       </c>
       <c r="E55">
-        <v>2.3566902</v>
+        <v>2.933116499999999</v>
       </c>
       <c r="F55">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G55">
-        <v>331</v>
+        <v>911</v>
       </c>
       <c r="H55">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -3301,28 +3349,34 @@
         <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C56" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="D56">
-        <v>49.8912963</v>
+        <v>49.7097598</v>
       </c>
       <c r="E56">
-        <v>2.3038483</v>
+        <v>2.773197300000001</v>
       </c>
       <c r="F56">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="G56">
+        <v>1068</v>
+      </c>
+      <c r="H56">
+        <v>2</v>
+      </c>
+      <c r="I56" t="b">
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -3330,34 +3384,34 @@
         <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C57" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="D57">
-        <v>49.8821619</v>
+        <v>49.8708087</v>
       </c>
       <c r="E57">
-        <v>2.3188738</v>
+        <v>2.5975248</v>
       </c>
       <c r="F57">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="G57">
-        <v>446</v>
+        <v>169</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -3365,34 +3419,34 @@
         <v>67</v>
       </c>
       <c r="B58" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C58" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="D58">
-        <v>49.9033033</v>
+        <v>49.7089958</v>
       </c>
       <c r="E58">
-        <v>2.3055391</v>
+        <v>2.773895500000001</v>
       </c>
       <c r="F58">
-        <v>4.4</v>
+        <v>3.8</v>
       </c>
       <c r="G58">
-        <v>99</v>
+        <v>831</v>
       </c>
       <c r="H58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -3400,31 +3454,34 @@
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C59" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="D59">
-        <v>49.8918596</v>
+        <v>49.6995639</v>
       </c>
       <c r="E59">
-        <v>2.309983700000001</v>
+        <v>2.7944886</v>
       </c>
       <c r="F59">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G59">
-        <v>108</v>
+        <v>175</v>
+      </c>
+      <c r="H59">
+        <v>2</v>
       </c>
       <c r="I59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -3432,28 +3489,34 @@
         <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C60" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D60">
-        <v>49.8924005</v>
+        <v>50.1980106</v>
       </c>
       <c r="E60">
-        <v>2.308677899999999</v>
+        <v>2.8759627</v>
       </c>
       <c r="F60">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>82</v>
+      </c>
+      <c r="H60">
+        <v>1</v>
+      </c>
+      <c r="I60" t="b">
+        <v>0</v>
       </c>
       <c r="J60" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -3461,31 +3524,31 @@
         <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C61" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="D61">
-        <v>49.88939339999999</v>
+        <v>49.6978505</v>
       </c>
       <c r="E61">
-        <v>2.3103845</v>
+        <v>2.791623399999999</v>
       </c>
       <c r="F61">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="G61">
-        <v>170</v>
+        <v>201</v>
       </c>
       <c r="I61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -3493,34 +3556,31 @@
         <v>71</v>
       </c>
       <c r="B62" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C62" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="D62">
-        <v>49.41652569999999</v>
+        <v>50.17135099999999</v>
       </c>
       <c r="E62">
-        <v>2.8255822</v>
+        <v>2.6318673</v>
       </c>
       <c r="F62">
-        <v>4.5</v>
+        <v>4.9</v>
       </c>
       <c r="G62">
-        <v>367</v>
-      </c>
-      <c r="H62">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="I62" t="b">
         <v>0</v>
       </c>
       <c r="J62" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="63" spans="1:11">
@@ -3528,34 +3588,31 @@
         <v>72</v>
       </c>
       <c r="B63" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C63" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D63">
-        <v>49.35251799999999</v>
+        <v>50.0034562</v>
       </c>
       <c r="E63">
-        <v>2.767293</v>
+        <v>2.911265</v>
       </c>
       <c r="F63">
-        <v>4.8</v>
+        <v>3.5</v>
       </c>
       <c r="G63">
-        <v>1246</v>
-      </c>
-      <c r="H63">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I63" t="b">
         <v>0</v>
       </c>
       <c r="J63" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
     </row>
     <row r="64" spans="1:11">
@@ -3563,34 +3620,34 @@
         <v>73</v>
       </c>
       <c r="B64" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C64" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="D64">
-        <v>49.64668830000001</v>
+        <v>49.6905687</v>
       </c>
       <c r="E64">
-        <v>2.56774</v>
+        <v>2.788442</v>
       </c>
       <c r="F64">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="G64">
-        <v>401</v>
+        <v>221</v>
       </c>
       <c r="H64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I64" t="b">
         <v>0</v>
       </c>
       <c r="J64" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -3598,34 +3655,31 @@
         <v>74</v>
       </c>
       <c r="B65" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C65" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="D65">
-        <v>49.4181602</v>
+        <v>49.7447927</v>
       </c>
       <c r="E65">
-        <v>2.8260746</v>
+        <v>3.0752862</v>
       </c>
       <c r="F65">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="G65">
-        <v>95</v>
-      </c>
-      <c r="H65">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="I65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
     </row>
     <row r="66" spans="1:11">
@@ -3633,31 +3687,34 @@
         <v>75</v>
       </c>
       <c r="B66" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C66" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D66">
-        <v>49.2062605</v>
+        <v>49.41652569999999</v>
       </c>
       <c r="E66">
-        <v>2.5796583</v>
+        <v>2.8255822</v>
       </c>
       <c r="F66">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="G66">
-        <v>321</v>
+        <v>367</v>
+      </c>
+      <c r="H66">
+        <v>2</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="67" spans="1:11">
@@ -3665,34 +3722,34 @@
         <v>76</v>
       </c>
       <c r="B67" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C67" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="D67">
-        <v>49.32945489999999</v>
+        <v>49.35251799999999</v>
       </c>
       <c r="E67">
-        <v>2.465046000000001</v>
+        <v>2.767293</v>
       </c>
       <c r="F67">
-        <v>3.7</v>
+        <v>4.8</v>
       </c>
       <c r="G67">
-        <v>140</v>
+        <v>1247</v>
       </c>
       <c r="H67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
     </row>
     <row r="68" spans="1:11">
@@ -3700,34 +3757,34 @@
         <v>77</v>
       </c>
       <c r="B68" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C68" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="D68">
-        <v>49.32898950000001</v>
+        <v>49.64668830000001</v>
       </c>
       <c r="E68">
-        <v>2.4629503</v>
+        <v>2.56774</v>
       </c>
       <c r="F68">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="G68">
-        <v>616</v>
+        <v>401</v>
       </c>
       <c r="H68">
         <v>1</v>
       </c>
       <c r="I68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -3735,34 +3792,34 @@
         <v>78</v>
       </c>
       <c r="B69" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C69" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D69">
-        <v>49.4786609</v>
+        <v>49.4181602</v>
       </c>
       <c r="E69">
-        <v>2.8784628</v>
+        <v>2.8260746</v>
       </c>
       <c r="F69">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="G69">
-        <v>544</v>
+        <v>95</v>
       </c>
       <c r="H69">
         <v>2</v>
       </c>
       <c r="I69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -3770,34 +3827,31 @@
         <v>79</v>
       </c>
       <c r="B70" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C70" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="D70">
-        <v>49.3854719</v>
+        <v>49.2062605</v>
       </c>
       <c r="E70">
-        <v>2.777325000000001</v>
+        <v>2.5796583</v>
       </c>
       <c r="F70">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="G70">
-        <v>777</v>
-      </c>
-      <c r="H70">
-        <v>2</v>
+        <v>321</v>
       </c>
       <c r="I70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -3805,31 +3859,34 @@
         <v>80</v>
       </c>
       <c r="B71" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C71" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="D71">
-        <v>49.398555</v>
+        <v>49.32945489999999</v>
       </c>
       <c r="E71">
-        <v>2.7974006</v>
+        <v>2.465046000000001</v>
       </c>
       <c r="F71">
-        <v>4.1</v>
+        <v>3.7</v>
       </c>
       <c r="G71">
-        <v>117</v>
+        <v>140</v>
+      </c>
+      <c r="H71">
+        <v>1</v>
       </c>
       <c r="I71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -3837,34 +3894,34 @@
         <v>81</v>
       </c>
       <c r="B72" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C72" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D72">
-        <v>49.551745</v>
+        <v>49.32898950000001</v>
       </c>
       <c r="E72">
-        <v>2.520455</v>
+        <v>2.4629503</v>
       </c>
       <c r="F72">
         <v>4.6</v>
       </c>
       <c r="G72">
-        <v>147</v>
+        <v>616</v>
       </c>
       <c r="H72">
         <v>1</v>
       </c>
       <c r="I72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -3872,34 +3929,34 @@
         <v>82</v>
       </c>
       <c r="B73" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C73" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D73">
-        <v>49.3084</v>
+        <v>49.4786609</v>
       </c>
       <c r="E73">
-        <v>2.728939</v>
+        <v>2.8784628</v>
       </c>
       <c r="F73">
         <v>4.4</v>
       </c>
       <c r="G73">
-        <v>460</v>
+        <v>545</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -3907,31 +3964,34 @@
         <v>83</v>
       </c>
       <c r="B74" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C74" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D74">
-        <v>49.4260495</v>
+        <v>49.3854719</v>
       </c>
       <c r="E74">
-        <v>2.6380979</v>
+        <v>2.777325000000001</v>
       </c>
       <c r="F74">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="G74">
-        <v>209</v>
+        <v>777</v>
+      </c>
+      <c r="H74">
+        <v>2</v>
       </c>
       <c r="I74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
     </row>
     <row r="75" spans="1:11">
@@ -3939,34 +3999,31 @@
         <v>84</v>
       </c>
       <c r="B75" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C75" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D75">
-        <v>49.4171323</v>
+        <v>49.398555</v>
       </c>
       <c r="E75">
-        <v>2.826151</v>
+        <v>2.7974006</v>
       </c>
       <c r="F75">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="G75">
-        <v>1419</v>
-      </c>
-      <c r="H75">
-        <v>2</v>
+        <v>117</v>
       </c>
       <c r="I75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -3974,34 +4031,34 @@
         <v>85</v>
       </c>
       <c r="B76" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C76" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="D76">
-        <v>49.4888858</v>
+        <v>49.551745</v>
       </c>
       <c r="E76">
-        <v>2.8153957</v>
+        <v>2.520455</v>
       </c>
       <c r="F76">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="G76">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="H76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
     </row>
     <row r="77" spans="1:11">
@@ -4009,22 +4066,22 @@
         <v>86</v>
       </c>
       <c r="B77" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C77" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="D77">
-        <v>49.4291534</v>
+        <v>49.3084</v>
       </c>
       <c r="E77">
-        <v>2.8386883</v>
+        <v>2.728939</v>
       </c>
       <c r="F77">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="G77">
-        <v>81</v>
+        <v>460</v>
       </c>
       <c r="H77">
         <v>1</v>
@@ -4033,10 +4090,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="K77" s="2" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
     </row>
     <row r="78" spans="1:11">
@@ -4044,31 +4101,31 @@
         <v>87</v>
       </c>
       <c r="B78" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C78" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D78">
-        <v>49.4219351</v>
+        <v>49.4260495</v>
       </c>
       <c r="E78">
-        <v>2.8431248</v>
+        <v>2.6380979</v>
       </c>
       <c r="F78">
         <v>4.4</v>
       </c>
       <c r="G78">
-        <v>197</v>
-      </c>
-      <c r="H78">
+        <v>209</v>
+      </c>
+      <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="K78" s="2" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
     </row>
     <row r="79" spans="1:11">
@@ -4076,31 +4133,34 @@
         <v>88</v>
       </c>
       <c r="B79" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C79" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="D79">
-        <v>49.416086</v>
+        <v>49.4171323</v>
       </c>
       <c r="E79">
-        <v>2.819035</v>
+        <v>2.826151</v>
       </c>
       <c r="F79">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="G79">
-        <v>114</v>
+        <v>1419</v>
+      </c>
+      <c r="H79">
+        <v>2</v>
       </c>
       <c r="I79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
     </row>
     <row r="80" spans="1:11">
@@ -4108,34 +4168,34 @@
         <v>89</v>
       </c>
       <c r="B80" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C80" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="D80">
-        <v>49.4057464</v>
+        <v>49.4888858</v>
       </c>
       <c r="E80">
-        <v>2.7834179</v>
+        <v>2.8153957</v>
       </c>
       <c r="F80">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="G80">
-        <v>4036</v>
+        <v>142</v>
       </c>
       <c r="H80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="K80" s="2" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
     </row>
     <row r="81" spans="1:11">
@@ -4143,34 +4203,34 @@
         <v>90</v>
       </c>
       <c r="B81" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C81" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="D81">
-        <v>49.4054683</v>
+        <v>49.4291534</v>
       </c>
       <c r="E81">
-        <v>2.7843017</v>
+        <v>2.8386883</v>
       </c>
       <c r="F81">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="G81">
-        <v>5354</v>
+        <v>81</v>
       </c>
       <c r="H81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J81" t="s">
-        <v>254</v>
+        <v>268</v>
       </c>
       <c r="K81" s="2" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -4178,34 +4238,168 @@
         <v>91</v>
       </c>
       <c r="B82" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C82" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="D82">
+        <v>49.4219351</v>
+      </c>
+      <c r="E82">
+        <v>2.8431248</v>
+      </c>
+      <c r="F82">
+        <v>4.4</v>
+      </c>
+      <c r="G82">
+        <v>197</v>
+      </c>
+      <c r="H82">
+        <v>1</v>
+      </c>
+      <c r="J82" t="s">
+        <v>268</v>
+      </c>
+      <c r="K82" s="2" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11">
+      <c r="A83" t="s">
+        <v>92</v>
+      </c>
+      <c r="B83" t="s">
+        <v>177</v>
+      </c>
+      <c r="C83" t="s">
+        <v>262</v>
+      </c>
+      <c r="D83">
+        <v>49.416086</v>
+      </c>
+      <c r="E83">
+        <v>2.819035</v>
+      </c>
+      <c r="F83">
+        <v>4.2</v>
+      </c>
+      <c r="G83">
+        <v>114</v>
+      </c>
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" t="s">
+        <v>268</v>
+      </c>
+      <c r="K83" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11">
+      <c r="A84" t="s">
+        <v>93</v>
+      </c>
+      <c r="B84" t="s">
+        <v>178</v>
+      </c>
+      <c r="C84" t="s">
+        <v>263</v>
+      </c>
+      <c r="D84">
+        <v>49.4057464</v>
+      </c>
+      <c r="E84">
+        <v>2.7834179</v>
+      </c>
+      <c r="F84">
+        <v>4.2</v>
+      </c>
+      <c r="G84">
+        <v>4038</v>
+      </c>
+      <c r="H84">
+        <v>1</v>
+      </c>
+      <c r="I84" t="b">
+        <v>1</v>
+      </c>
+      <c r="J84" t="s">
+        <v>268</v>
+      </c>
+      <c r="K84" s="2" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11">
+      <c r="A85" t="s">
+        <v>94</v>
+      </c>
+      <c r="B85" t="s">
+        <v>179</v>
+      </c>
+      <c r="C85" t="s">
+        <v>264</v>
+      </c>
+      <c r="D85">
+        <v>49.4054683</v>
+      </c>
+      <c r="E85">
+        <v>2.7843017</v>
+      </c>
+      <c r="F85">
+        <v>4.1</v>
+      </c>
+      <c r="G85">
+        <v>5356</v>
+      </c>
+      <c r="H85">
+        <v>2</v>
+      </c>
+      <c r="I85" t="b">
+        <v>1</v>
+      </c>
+      <c r="J85" t="s">
+        <v>268</v>
+      </c>
+      <c r="K85" s="2" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11">
+      <c r="A86" t="s">
+        <v>95</v>
+      </c>
+      <c r="B86" t="s">
+        <v>180</v>
+      </c>
+      <c r="C86" t="s">
+        <v>265</v>
+      </c>
+      <c r="D86">
         <v>49.39665679999999</v>
       </c>
-      <c r="E82">
+      <c r="E86">
         <v>2.786974299999999</v>
       </c>
-      <c r="F82">
+      <c r="F86">
         <v>3.9</v>
       </c>
-      <c r="G82">
+      <c r="G86">
         <v>154</v>
       </c>
-      <c r="H82">
-        <v>2</v>
-      </c>
-      <c r="I82" t="b">
-        <v>0</v>
-      </c>
-      <c r="J82" t="s">
-        <v>254</v>
-      </c>
-      <c r="K82" s="2" t="s">
-        <v>337</v>
+      <c r="H86">
+        <v>2</v>
+      </c>
+      <c r="I86" t="b">
+        <v>1</v>
+      </c>
+      <c r="J86" t="s">
+        <v>268</v>
+      </c>
+      <c r="K86" s="2" t="s">
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -4291,6 +4485,10 @@
     <hyperlink ref="K80" r:id="rId79"/>
     <hyperlink ref="K81" r:id="rId80"/>
     <hyperlink ref="K82" r:id="rId81"/>
+    <hyperlink ref="K83" r:id="rId82"/>
+    <hyperlink ref="K84" r:id="rId83"/>
+    <hyperlink ref="K85" r:id="rId84"/>
+    <hyperlink ref="K86" r:id="rId85"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
optimized pipeline by dropping big city centres
</commit_message>
<xml_diff>
--- a/data/processed/candidates.xlsx
+++ b/data/processed/candidates.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="257">
   <si>
     <t>place_id</t>
   </si>
@@ -55,72 +55,18 @@
     <t>ChIJ6U6ntWgUw0cRZrq8q_ohqUU</t>
   </si>
   <si>
-    <t>ChIJaccB1UBxw0cRocMTI7DALgE</t>
-  </si>
-  <si>
-    <t>ChIJd92M2UBxw0cRcLC_XWtAw5M</t>
-  </si>
-  <si>
-    <t>ChIJcw76AERxw0cRCZ9UPLL7szA</t>
-  </si>
-  <si>
-    <t>ChIJfXFDIWBxw0cRE9YYAtd17F4</t>
-  </si>
-  <si>
     <t>ChIJYdFddZ1nw0cRf0zN9IQqQ7Q</t>
   </si>
   <si>
-    <t>ChIJXRIrlEBxw0cRsx0RGjb2Ggw</t>
-  </si>
-  <si>
-    <t>ChIJ66An1k1xw0cRrkKcb_6Z488</t>
-  </si>
-  <si>
     <t>ChIJl4CsVsF2w0cRytpeXShIbNE</t>
   </si>
   <si>
-    <t>ChIJI46pG0dxw0cRIXbgTe31oZc</t>
-  </si>
-  <si>
-    <t>ChIJvwaiZ1pxw0cRITmiV6KwtPw</t>
-  </si>
-  <si>
-    <t>ChIJY61l4kNxw0cRcr5s10LzLuM</t>
-  </si>
-  <si>
-    <t>ChIJZ6VMYFdxw0cRfVoCvTscwOg</t>
-  </si>
-  <si>
-    <t>ChIJl8_4Z05xw0cRY8fapfMJrxc</t>
-  </si>
-  <si>
     <t>ChIJr82_7G1yw0cRebseGTV57d0</t>
   </si>
   <si>
-    <t>ChIJD8S0YEdxw0cRfVs16dksyJQ</t>
-  </si>
-  <si>
     <t>ChIJi-zbr0UQw0cRyBDtc11VPiE</t>
   </si>
   <si>
-    <t>ChIJyXZkekZxw0cRb9uqej8bxZY</t>
-  </si>
-  <si>
-    <t>ChIJs0g1-kZxw0cR46lPwxTdOpg</t>
-  </si>
-  <si>
-    <t>ChIJU1sJSUZxw0cRgmHC8o3MZwQ</t>
-  </si>
-  <si>
-    <t>ChIJ0X-9015xw0cRsPLuG79Kn4s</t>
-  </si>
-  <si>
-    <t>ChIJO5B6a0Zxw0cRCSaWrQEL7bE</t>
-  </si>
-  <si>
-    <t>ChIJW3OtxDlxw0cRM_nXQaujiBg</t>
-  </si>
-  <si>
     <t>ChIJmzeJyjnWwkcRCMoN538F2as</t>
   </si>
   <si>
@@ -130,18 +76,12 @@
     <t>ChIJ2y_9XsbS3EcRhE397G30AOw</t>
   </si>
   <si>
-    <t>ChIJR02hQ3gqw0cRYYmLHgPR0D8</t>
-  </si>
-  <si>
     <t>ChIJ-3DxCUkww0cRGMRoItLlQSk</t>
   </si>
   <si>
     <t>ChIJX7J7eBQkw0cR7A93qiQYvLY</t>
   </si>
   <si>
-    <t>ChIJCQOYnYjVwkcR6lYaR-xTg98</t>
-  </si>
-  <si>
     <t>ChIJn9OLi97fwkcRN9zVioh1KUc</t>
   </si>
   <si>
@@ -151,9 +91,6 @@
     <t>ChIJiXvXemrWwkcR1Th5LFqOW7s</t>
   </si>
   <si>
-    <t>ChIJb-2V4XYqw0cRcdf1yjoy0F8</t>
-  </si>
-  <si>
     <t>ChIJbx9ih_Aw3UcRoGOf2o5HMr4</t>
   </si>
   <si>
@@ -241,18 +178,12 @@
     <t>ChIJVToX4xIO6EcRcQvXHvdfhpA</t>
   </si>
   <si>
-    <t>ChIJ3fl0IYHW50cR_mvDeqFjsfs</t>
-  </si>
-  <si>
     <t>ChIJ8fv7gmfT50cRw_C5VLq33bw</t>
   </si>
   <si>
     <t>ChIJ-yBXGjTA50cRvodrnqP-iM4</t>
   </si>
   <si>
-    <t>ChIJnenC2IbW50cRkD8sVzSdwis</t>
-  </si>
-  <si>
     <t>ChIJV7sjxtIw5kcRv54y3LHxHeo</t>
   </si>
   <si>
@@ -280,9 +211,6 @@
     <t>ChIJvTGf7YXO50cRnwZKFYhbTls</t>
   </si>
   <si>
-    <t>ChIJcdBu1YDW50cRP2FmSx9Z-8Y</t>
-  </si>
-  <si>
     <t>ChIJh0hyKGHX50cRc0uHq15o8sg</t>
   </si>
   <si>
@@ -310,72 +238,18 @@
     <t>Hof van Cleve</t>
   </si>
   <si>
-    <t>De Witte Leeuw | Gent</t>
-  </si>
-  <si>
-    <t>Korenlei Twee</t>
-  </si>
-  <si>
-    <t>Lucy Chang Gent</t>
-  </si>
-  <si>
-    <t>Café Parti</t>
-  </si>
-  <si>
     <t>'t Brigandje</t>
   </si>
   <si>
-    <t>De Gekroonde Hoofden</t>
-  </si>
-  <si>
-    <t>faim fatale</t>
-  </si>
-  <si>
     <t>LAGO Gent Rozebroeken</t>
   </si>
   <si>
-    <t>Amatsu</t>
-  </si>
-  <si>
-    <t>Firenze</t>
-  </si>
-  <si>
-    <t>JACQUELINE</t>
-  </si>
-  <si>
-    <t>Prima Donna</t>
-  </si>
-  <si>
-    <t>Martino</t>
-  </si>
-  <si>
     <t>Brasserie Latem</t>
   </si>
   <si>
-    <t>Il Cortile 🇮🇹</t>
-  </si>
-  <si>
     <t>'t Veer</t>
   </si>
   <si>
-    <t>Maximiliaan</t>
-  </si>
-  <si>
-    <t>Amadeus Gent 2 - Belfort</t>
-  </si>
-  <si>
-    <t>Tokyo Sushi Ghent</t>
-  </si>
-  <si>
-    <t>Jan van den Bon</t>
-  </si>
-  <si>
-    <t>'t Vosken</t>
-  </si>
-  <si>
-    <t>MULTATULI</t>
-  </si>
-  <si>
     <t>Friterie de l'Hôtel de Ville</t>
   </si>
   <si>
@@ -385,18 +259,12 @@
     <t>Ice Mountain Adventure Park</t>
   </si>
   <si>
-    <t>In Bocca Al Lupo</t>
-  </si>
-  <si>
     <t>Vijverhof</t>
   </si>
   <si>
     <t>Ferme Balthazar</t>
   </si>
   <si>
-    <t>Bouillon De La Paix</t>
-  </si>
-  <si>
     <t>ADANA</t>
   </si>
   <si>
@@ -406,9 +274,6 @@
     <t>KFC Lilles Lezennes</t>
   </si>
   <si>
-    <t>Estaminet Chez La Vieille</t>
-  </si>
-  <si>
     <t>La Fiesta</t>
   </si>
   <si>
@@ -496,18 +361,12 @@
     <t>Pizza Anna</t>
   </si>
   <si>
-    <t>Le Stromboli</t>
-  </si>
-  <si>
     <t>A l'Auberge du Bac</t>
   </si>
   <si>
     <t>EGEE</t>
   </si>
   <si>
-    <t>Restaurant L'endroit</t>
-  </si>
-  <si>
     <t>LE JULIANON</t>
   </si>
   <si>
@@ -535,9 +394,6 @@
     <t>La Pause Pizza</t>
   </si>
   <si>
-    <t>Restaurant Compiegne - Soprano</t>
-  </si>
-  <si>
     <t>Restaurant La Bergerie</t>
   </si>
   <si>
@@ -565,72 +421,18 @@
     <t>Riemegemstraat 1, Kruisem</t>
   </si>
   <si>
-    <t>Graslei 6, Gent</t>
-  </si>
-  <si>
-    <t>Korenlei 2, Gent</t>
-  </si>
-  <si>
-    <t>Jakobijnenstraat 1, Gent</t>
-  </si>
-  <si>
-    <t>Koningin Maria Hendrikaplein 65A, Gent</t>
-  </si>
-  <si>
     <t>Urselweg 100, Maldegem</t>
   </si>
   <si>
-    <t>Burgstraat 4, Gent</t>
-  </si>
-  <si>
-    <t>Zuidstationstraat 14, Gent</t>
-  </si>
-  <si>
     <t>Victor Braeckmanlaan 180/B, Gent</t>
   </si>
   <si>
-    <t>Nederkouter 139, Gent</t>
-  </si>
-  <si>
-    <t>Sint-Amandstraat 1, Gent</t>
-  </si>
-  <si>
-    <t>Jakobijnenstraat 12, Gent</t>
-  </si>
-  <si>
-    <t>Overpoortstraat 46, Gent</t>
-  </si>
-  <si>
-    <t>Vlaanderenstraat 125, Gent</t>
-  </si>
-  <si>
     <t>Kortrijksesteenweg 9, Sint-Martens-Latem</t>
   </si>
   <si>
-    <t>Kraanlei 53, Gent</t>
-  </si>
-  <si>
     <t>Berchemweg 191, Oudenaarde</t>
   </si>
   <si>
-    <t>Mageleinstraat 50, Gent</t>
-  </si>
-  <si>
-    <t>Goudenleeuwplein 7, Gent</t>
-  </si>
-  <si>
-    <t>Botermarkt 10, Gent</t>
-  </si>
-  <si>
-    <t>Floraliënlaan 22, Gent</t>
-  </si>
-  <si>
-    <t>Sint-Baafsplein 19, Gent</t>
-  </si>
-  <si>
-    <t>Huidevetterskaai 40, Gent</t>
-  </si>
-  <si>
     <t>Place Van Gogh, Villeneuve-d'Ascq</t>
   </si>
   <si>
@@ -640,18 +442,12 @@
     <t>Rue des Rubaniers 7780, Comines-Warneton</t>
   </si>
   <si>
-    <t>1 Rue des Vieux Murs, Lille</t>
-  </si>
-  <si>
     <t>Marremstraat 3, Wevelgem</t>
   </si>
   <si>
     <t>Drève des Préaches 4, Mouscron</t>
   </si>
   <si>
-    <t>25 Place Rihour, Lille</t>
-  </si>
-  <si>
     <t>Rue Dorez 15, Tournai</t>
   </si>
   <si>
@@ -661,9 +457,6 @@
     <t>Rue de Chanzy - Lezennes, Lezennes</t>
   </si>
   <si>
-    <t>60 Rue de Gand, Lille</t>
-  </si>
-  <si>
     <t>102 Boulevard Emile Basly, Lens</t>
   </si>
   <si>
@@ -751,18 +544,12 @@
     <t>45 Rue du Général Leclerc, Ham</t>
   </si>
   <si>
-    <t>Accès, 12 Rue des Cordeliers, 2 Rue des Lombards, Compiègne</t>
-  </si>
-  <si>
     <t>1 Quai d'Estienne d'Orves, Lacroix-Saint-Ouen</t>
   </si>
   <si>
     <t>1 Rue Parmentier, Montdidier</t>
   </si>
   <si>
-    <t>14 Rue des Pâtissiers, Compiègne</t>
-  </si>
-  <si>
     <t>5 Place Gérard de Nerval, Senlis</t>
   </si>
   <si>
@@ -790,9 +577,6 @@
     <t>62 Avenue de Flandre, Estrées-Saint-Denis</t>
   </si>
   <si>
-    <t>22 Rue Jean Legendre, Compiègne</t>
-  </si>
-  <si>
     <t>10 Allée des Platanes, Villers-sur-Coudun</t>
   </si>
   <si>
@@ -817,10 +601,7 @@
     <t>restaurant, food, point_of_interest, establishment</t>
   </si>
   <si>
-    <t>restaurant, health, food, point_of_interest, establishment</t>
-  </si>
-  <si>
-    <t>restaurant, point_of_interest, food, establishment</t>
+    <t>health, restaurant, food, point_of_interest, establishment</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.8354964,3.3953747&amp;query_place_id=ChIJv8_dynU9w0cRPwuu4Hw6BCM</t>
@@ -829,72 +610,18 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.9036673,3.5096569&amp;query_place_id=ChIJ6U6ntWgUw0cRZrq8q_ohqUU</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0551243,3.721278300000001&amp;query_place_id=ChIJaccB1UBxw0cRocMTI7DALgE</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.05561119999999,3.7205134&amp;query_place_id=ChIJd92M2UBxw0cRcLC_XWtAw5M</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0521389,3.7201179&amp;query_place_id=ChIJcw76AERxw0cRCZ9UPLL7szA</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0372949,3.7103165&amp;query_place_id=ChIJfXFDIWBxw0cRE9YYAtd17F4</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.16801830000001,3.4724922&amp;query_place_id=ChIJYdFddZ1nw0cRf0zN9IQqQ7Q</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0567995,3.7196267&amp;query_place_id=ChIJXRIrlEBxw0cRsx0RGjb2Ggw</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0490043,3.732778999999999&amp;query_place_id=ChIJ66An1k1xw0cRrkKcb_6Z488</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0595473,3.761043&amp;query_place_id=ChIJl4CsVsF2w0cRytpeXShIbNE</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0465092,3.7225456&amp;query_place_id=ChIJI46pG0dxw0cRIXbgTe31oZc</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0438889,3.7247222&amp;query_place_id=ChIJvwaiZ1pxw0cRITmiV6KwtPw</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0522725,3.7198882&amp;query_place_id=ChIJY61l4kNxw0cRcr5s10LzLuM</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0403269,3.725390500000001&amp;query_place_id=ChIJZ6VMYFdxw0cRfVoCvTscwOg</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.04891989999999,3.7312643&amp;query_place_id=ChIJl8_4Z05xw0cRY8fapfMJrxc</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=51.0140263,3.6491051&amp;query_place_id=ChIJr82_7G1yw0cRebseGTV57d0</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.05728250000001,3.7231798&amp;query_place_id=ChIJD8S0YEdxw0cRfVs16dksyJQ</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.81935849999999,3.5751952&amp;query_place_id=ChIJi-zbr0UQw0cRyBDtc11VPiE</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.052705,3.724562499999999&amp;query_place_id=ChIJyXZkekZxw0cRb9uqej8bxZY</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.05421639999999,3.7240936&amp;query_place_id=ChIJs0g1-kZxw0cR46lPwxTdOpg</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.0540422,3.7255715&amp;query_place_id=ChIJU1sJSUZxw0cRgmHC8o3MZwQ</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.03981009999999,3.718738&amp;query_place_id=ChIJ0X-9015xw0cRsPLuG79Kn4s</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.05352310000001,3.726121400000001&amp;query_place_id=ChIJO5B6a0Zxw0cRCSaWrQEL7bE</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=51.061058,3.72782&amp;query_place_id=ChIJW3OtxDlxw0cRM_nXQaujiBg</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.61939779999999,3.132437599999999&amp;query_place_id=ChIJmzeJyjnWwkcRCMoN538F2as</t>
   </si>
   <si>
@@ -904,18 +631,12 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.78213179999999,3.0023986&amp;query_place_id=ChIJ2y_9XsbS3EcRhE397G30AOw</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.64078540000001,3.061416099999999&amp;query_place_id=ChIJR02hQ3gqw0cRYYmLHgPR0D8</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.8263743,3.1773917&amp;query_place_id=ChIJ-3DxCUkww0cRGMRoItLlQSk</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.7344444,3.2863889&amp;query_place_id=ChIJX7J7eBQkw0cR7A93qiQYvLY</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.63577600000001,3.0634036&amp;query_place_id=ChIJCQOYnYjVwkcR6lYaR-xTg98</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.606813,3.382719799999999&amp;query_place_id=ChIJn9OLi97fwkcRN9zVioh1KUc</t>
   </si>
   <si>
@@ -925,9 +646,6 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.61273699999999,3.123373&amp;query_place_id=ChIJiXvXemrWwkcR1Th5LFqOW7s</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=50.6427316,3.0668892&amp;query_place_id=ChIJb-2V4XYqw0cRcdf1yjoy0F8</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=50.43022910000001,2.8241761&amp;query_place_id=ChIJbx9ih_Aw3UcRoGOf2o5HMr4</t>
   </si>
   <si>
@@ -1015,18 +733,12 @@
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.7447927,3.0752862&amp;query_place_id=ChIJVToX4xIO6EcRcQvXHvdfhpA</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.41652569999999,2.8255822&amp;query_place_id=ChIJ3fl0IYHW50cR_mvDeqFjsfs</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.35251799999999,2.767293&amp;query_place_id=ChIJ8fv7gmfT50cRw_C5VLq33bw</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.64668830000001,2.56774&amp;query_place_id=ChIJ-yBXGjTA50cRvodrnqP-iM4</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.4181602,2.8260746&amp;query_place_id=ChIJnenC2IbW50cRkD8sVzSdwis</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.2062605,2.5796583&amp;query_place_id=ChIJV7sjxtIw5kcRv54y3LHxHeo</t>
   </si>
   <si>
@@ -1052,9 +764,6 @@
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.4260495,2.6380979&amp;query_place_id=ChIJvTGf7YXO50cRnwZKFYhbTls</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/search/?api=1&amp;query=49.4171323,2.826151&amp;query_place_id=ChIJcdBu1YDW50cRP2FmSx9Z-8Y</t>
   </si>
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=49.4888858,2.8153957&amp;query_place_id=ChIJh0hyKGHX50cRc0uHq15o8sg</t>
@@ -1446,7 +1155,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K86"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -1489,10 +1198,10 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>181</v>
+        <v>133</v>
       </c>
       <c r="D2">
         <v>50.8354964</v>
@@ -1513,10 +1222,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>269</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1524,10 +1233,10 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>182</v>
+        <v>134</v>
       </c>
       <c r="D3">
         <v>50.9036673</v>
@@ -1545,13 +1254,13 @@
         <v>4</v>
       </c>
       <c r="I3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>270</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1559,34 +1268,34 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>183</v>
+        <v>135</v>
       </c>
       <c r="D4">
-        <v>51.0551243</v>
+        <v>51.16801830000001</v>
       </c>
       <c r="E4">
-        <v>3.721278300000001</v>
+        <v>3.4724922</v>
       </c>
       <c r="F4">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="G4">
-        <v>1552</v>
+        <v>758</v>
       </c>
       <c r="H4">
         <v>2</v>
       </c>
       <c r="I4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>271</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1594,34 +1303,31 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>184</v>
+        <v>136</v>
       </c>
       <c r="D5">
-        <v>51.05561119999999</v>
+        <v>51.0595473</v>
       </c>
       <c r="E5">
-        <v>3.7205134</v>
+        <v>3.761043</v>
       </c>
       <c r="F5">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>525</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
+        <v>6396</v>
       </c>
       <c r="I5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>266</v>
+        <v>195</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>272</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1629,34 +1335,34 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>185</v>
+        <v>137</v>
       </c>
       <c r="D6">
-        <v>51.0521389</v>
+        <v>51.0140263</v>
       </c>
       <c r="E6">
-        <v>3.7201179</v>
+        <v>3.6491051</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>4.4</v>
       </c>
       <c r="G6">
-        <v>1311</v>
+        <v>412</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" t="b">
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>273</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1664,34 +1370,34 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>186</v>
+        <v>138</v>
       </c>
       <c r="D7">
-        <v>51.0372949</v>
+        <v>50.81935849999999</v>
       </c>
       <c r="E7">
-        <v>3.7103165</v>
+        <v>3.5751952</v>
       </c>
       <c r="F7">
         <v>4.3</v>
       </c>
       <c r="G7">
-        <v>683</v>
+        <v>925</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7" t="b">
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>274</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1699,34 +1405,31 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
-        <v>187</v>
+        <v>139</v>
       </c>
       <c r="D8">
-        <v>51.16801830000001</v>
+        <v>50.61939779999999</v>
       </c>
       <c r="E8">
-        <v>3.4724922</v>
+        <v>3.132437599999999</v>
       </c>
       <c r="F8">
         <v>4.2</v>
       </c>
       <c r="G8">
-        <v>757</v>
-      </c>
-      <c r="H8">
-        <v>2</v>
+        <v>127</v>
       </c>
       <c r="I8" t="b">
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>275</v>
+        <v>202</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1734,34 +1437,34 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>188</v>
+        <v>140</v>
       </c>
       <c r="D9">
-        <v>51.0567995</v>
+        <v>50.8500201</v>
       </c>
       <c r="E9">
-        <v>3.7196267</v>
+        <v>2.881268900000001</v>
       </c>
       <c r="F9">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G9">
-        <v>2128</v>
+        <v>610</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>276</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1769,34 +1472,31 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
-        <v>189</v>
+        <v>141</v>
       </c>
       <c r="D10">
-        <v>51.0490043</v>
+        <v>50.78213179999999</v>
       </c>
       <c r="E10">
-        <v>3.732778999999999</v>
+        <v>3.0023986</v>
       </c>
       <c r="F10">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="G10">
-        <v>352</v>
-      </c>
-      <c r="H10">
-        <v>2</v>
+        <v>3498</v>
       </c>
       <c r="I10" t="b">
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>277</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1804,31 +1504,34 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>190</v>
+        <v>142</v>
       </c>
       <c r="D11">
-        <v>51.0595473</v>
+        <v>50.8263743</v>
       </c>
       <c r="E11">
-        <v>3.761043</v>
+        <v>3.1773917</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="G11">
-        <v>6396</v>
+        <v>661</v>
+      </c>
+      <c r="H11">
+        <v>2</v>
       </c>
       <c r="I11" t="b">
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>267</v>
+        <v>194</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>278</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1836,34 +1539,34 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="C12" t="s">
-        <v>191</v>
+        <v>143</v>
       </c>
       <c r="D12">
-        <v>51.0465092</v>
+        <v>50.7344444</v>
       </c>
       <c r="E12">
-        <v>3.7225456</v>
+        <v>3.2863889</v>
       </c>
       <c r="F12">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="G12">
-        <v>386</v>
+        <v>2984</v>
       </c>
       <c r="H12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I12" t="b">
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>279</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1871,34 +1574,34 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="C13" t="s">
-        <v>192</v>
+        <v>144</v>
       </c>
       <c r="D13">
-        <v>51.0438889</v>
+        <v>50.606813</v>
       </c>
       <c r="E13">
-        <v>3.7247222</v>
+        <v>3.382719799999999</v>
       </c>
       <c r="F13">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="G13">
-        <v>1103</v>
+        <v>599</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" t="b">
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>280</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1906,34 +1609,31 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="C14" t="s">
-        <v>193</v>
+        <v>145</v>
       </c>
       <c r="D14">
-        <v>51.0522725</v>
+        <v>50.5243349</v>
       </c>
       <c r="E14">
-        <v>3.7198882</v>
+        <v>3.0756846</v>
       </c>
       <c r="F14">
-        <v>4.1</v>
+        <v>4.4</v>
       </c>
       <c r="G14">
-        <v>348</v>
-      </c>
-      <c r="H14">
-        <v>2</v>
+        <v>124</v>
       </c>
       <c r="I14" t="b">
         <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>281</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1941,34 +1641,34 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="D15">
-        <v>51.0403269</v>
+        <v>50.61273699999999</v>
       </c>
       <c r="E15">
-        <v>3.725390500000001</v>
+        <v>3.123373</v>
       </c>
       <c r="F15">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
       <c r="G15">
-        <v>728</v>
+        <v>4178</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>282</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1976,34 +1676,31 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
-        <v>195</v>
+        <v>147</v>
       </c>
       <c r="D16">
-        <v>51.04891989999999</v>
+        <v>50.43022910000001</v>
       </c>
       <c r="E16">
-        <v>3.7312643</v>
+        <v>2.8241761</v>
       </c>
       <c r="F16">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="G16">
-        <v>308</v>
-      </c>
-      <c r="H16">
-        <v>2</v>
+        <v>430</v>
       </c>
       <c r="I16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>283</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -2011,34 +1708,34 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="C17" t="s">
-        <v>196</v>
+        <v>148</v>
       </c>
       <c r="D17">
-        <v>51.0140263</v>
+        <v>50.42831</v>
       </c>
       <c r="E17">
-        <v>3.6491051</v>
+        <v>2.826468599999999</v>
       </c>
       <c r="F17">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="G17">
-        <v>412</v>
+        <v>847</v>
       </c>
       <c r="H17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>284</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2046,34 +1743,34 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C18" t="s">
-        <v>197</v>
+        <v>149</v>
       </c>
       <c r="D18">
-        <v>51.05728250000001</v>
+        <v>50.2927725</v>
       </c>
       <c r="E18">
-        <v>3.7231798</v>
+        <v>2.780148199999999</v>
       </c>
       <c r="F18">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="G18">
-        <v>829</v>
+        <v>690</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18" t="b">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>285</v>
+        <v>212</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2081,34 +1778,28 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
-        <v>198</v>
+        <v>150</v>
       </c>
       <c r="D19">
-        <v>50.81935849999999</v>
+        <v>50.3472046</v>
       </c>
       <c r="E19">
-        <v>3.5751952</v>
+        <v>2.6535711</v>
       </c>
       <c r="F19">
-        <v>4.3</v>
+        <v>4.8</v>
       </c>
       <c r="G19">
-        <v>924</v>
-      </c>
-      <c r="H19">
-        <v>2</v>
-      </c>
-      <c r="I19" t="b">
-        <v>1</v>
+        <v>164</v>
       </c>
       <c r="J19" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>286</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2116,22 +1807,22 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>199</v>
+        <v>151</v>
       </c>
       <c r="D20">
-        <v>51.052705</v>
+        <v>50.4796752</v>
       </c>
       <c r="E20">
-        <v>3.724562499999999</v>
+        <v>3.237034299999999</v>
       </c>
       <c r="F20">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G20">
-        <v>870</v>
+        <v>473</v>
       </c>
       <c r="H20">
         <v>2</v>
@@ -2140,10 +1831,10 @@
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>287</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2151,22 +1842,22 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>200</v>
+        <v>152</v>
       </c>
       <c r="D21">
-        <v>51.05421639999999</v>
+        <v>50.367342</v>
       </c>
       <c r="E21">
-        <v>3.7240936</v>
+        <v>3.081729999999999</v>
       </c>
       <c r="F21">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="G21">
-        <v>3834</v>
+        <v>377</v>
       </c>
       <c r="H21">
         <v>2</v>
@@ -2175,10 +1866,10 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>288</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2186,22 +1877,22 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="C22" t="s">
-        <v>201</v>
+        <v>153</v>
       </c>
       <c r="D22">
-        <v>51.0540422</v>
+        <v>50.3691968</v>
       </c>
       <c r="E22">
-        <v>3.7255715</v>
+        <v>3.078329</v>
       </c>
       <c r="F22">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="G22">
-        <v>805</v>
+        <v>464</v>
       </c>
       <c r="H22">
         <v>2</v>
@@ -2210,10 +1901,10 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>289</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2221,31 +1912,34 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>202</v>
+        <v>154</v>
       </c>
       <c r="D23">
-        <v>51.03981009999999</v>
+        <v>50.2091985</v>
       </c>
       <c r="E23">
-        <v>3.718738</v>
+        <v>3.1905208</v>
       </c>
       <c r="F23">
-        <v>4.6</v>
+        <v>3.8</v>
       </c>
       <c r="G23">
-        <v>100</v>
+        <v>399</v>
+      </c>
+      <c r="H23">
+        <v>2</v>
       </c>
       <c r="I23" t="b">
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>290</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2253,22 +1947,22 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="C24" t="s">
-        <v>203</v>
+        <v>155</v>
       </c>
       <c r="D24">
-        <v>51.05352310000001</v>
+        <v>50.0990133</v>
       </c>
       <c r="E24">
-        <v>3.726121400000001</v>
+        <v>2.8551931</v>
       </c>
       <c r="F24">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="G24">
-        <v>2022</v>
+        <v>888</v>
       </c>
       <c r="H24">
         <v>2</v>
@@ -2277,10 +1971,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>291</v>
+        <v>218</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2288,22 +1982,22 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="C25" t="s">
-        <v>204</v>
+        <v>156</v>
       </c>
       <c r="D25">
-        <v>51.061058</v>
+        <v>50.0440674</v>
       </c>
       <c r="E25">
-        <v>3.72782</v>
+        <v>2.666995500000001</v>
       </c>
       <c r="F25">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="G25">
-        <v>1351</v>
+        <v>607</v>
       </c>
       <c r="H25">
         <v>2</v>
@@ -2312,10 +2006,10 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -2323,31 +2017,34 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="C26" t="s">
-        <v>205</v>
+        <v>157</v>
       </c>
       <c r="D26">
-        <v>50.61939779999999</v>
+        <v>49.9306446</v>
       </c>
       <c r="E26">
-        <v>3.132437599999999</v>
+        <v>2.9373479</v>
       </c>
       <c r="F26">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="G26">
-        <v>127</v>
+        <v>687</v>
+      </c>
+      <c r="H26">
+        <v>2</v>
       </c>
       <c r="I26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>293</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2355,34 +2052,34 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="C27" t="s">
-        <v>206</v>
+        <v>158</v>
       </c>
       <c r="D27">
-        <v>50.8500201</v>
+        <v>49.9294497</v>
       </c>
       <c r="E27">
-        <v>2.881268900000001</v>
+        <v>2.9385445</v>
       </c>
       <c r="F27">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="G27">
-        <v>610</v>
+        <v>341</v>
       </c>
       <c r="H27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>294</v>
+        <v>221</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2390,31 +2087,31 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>122</v>
+        <v>98</v>
       </c>
       <c r="C28" t="s">
-        <v>207</v>
+        <v>159</v>
       </c>
       <c r="D28">
-        <v>50.78213179999999</v>
+        <v>49.887574</v>
       </c>
       <c r="E28">
-        <v>3.0023986</v>
+        <v>2.837822</v>
       </c>
       <c r="F28">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="G28">
-        <v>3498</v>
+        <v>627</v>
       </c>
       <c r="I28" t="b">
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>295</v>
+        <v>222</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2422,34 +2119,31 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="C29" t="s">
-        <v>208</v>
+        <v>160</v>
       </c>
       <c r="D29">
-        <v>50.64078540000001</v>
+        <v>49.9157805</v>
       </c>
       <c r="E29">
-        <v>3.061416099999999</v>
+        <v>2.9340714</v>
       </c>
       <c r="F29">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="G29">
-        <v>519</v>
-      </c>
-      <c r="H29">
-        <v>2</v>
+        <v>138</v>
       </c>
       <c r="I29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>296</v>
+        <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2457,34 +2151,34 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="C30" t="s">
-        <v>209</v>
+        <v>161</v>
       </c>
       <c r="D30">
-        <v>50.8263743</v>
+        <v>49.812285</v>
       </c>
       <c r="E30">
-        <v>3.1773917</v>
+        <v>2.7008719</v>
       </c>
       <c r="F30">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="G30">
-        <v>660</v>
+        <v>90</v>
       </c>
       <c r="H30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>297</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2492,34 +2186,34 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="C31" t="s">
-        <v>210</v>
+        <v>162</v>
       </c>
       <c r="D31">
-        <v>50.7344444</v>
+        <v>49.9470246</v>
       </c>
       <c r="E31">
-        <v>3.2863889</v>
+        <v>3.1002615</v>
       </c>
       <c r="F31">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="G31">
-        <v>2984</v>
+        <v>183</v>
       </c>
       <c r="H31">
         <v>2</v>
       </c>
       <c r="I31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>298</v>
+        <v>225</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2527,22 +2221,22 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>102</v>
       </c>
       <c r="C32" t="s">
-        <v>211</v>
+        <v>163</v>
       </c>
       <c r="D32">
-        <v>50.63577600000001</v>
+        <v>49.9000698</v>
       </c>
       <c r="E32">
-        <v>3.0634036</v>
+        <v>2.5028801</v>
       </c>
       <c r="F32">
-        <v>3.8</v>
+        <v>4.5</v>
       </c>
       <c r="G32">
-        <v>1199</v>
+        <v>223</v>
       </c>
       <c r="H32">
         <v>2</v>
@@ -2551,10 +2245,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>299</v>
+        <v>226</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2562,34 +2256,34 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>103</v>
       </c>
       <c r="C33" t="s">
-        <v>212</v>
+        <v>164</v>
       </c>
       <c r="D33">
-        <v>50.606813</v>
+        <v>50.0409911</v>
       </c>
       <c r="E33">
-        <v>3.382719799999999</v>
+        <v>2.6686785</v>
       </c>
       <c r="F33">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="G33">
-        <v>598</v>
+        <v>584</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>300</v>
+        <v>227</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2597,31 +2291,34 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="C34" t="s">
-        <v>213</v>
+        <v>165</v>
       </c>
       <c r="D34">
-        <v>50.5243349</v>
+        <v>49.9291968</v>
       </c>
       <c r="E34">
-        <v>3.0756846</v>
+        <v>2.933116499999999</v>
       </c>
       <c r="F34">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="G34">
-        <v>124</v>
+        <v>913</v>
+      </c>
+      <c r="H34">
+        <v>2</v>
       </c>
       <c r="I34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>301</v>
+        <v>228</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2629,22 +2326,22 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>129</v>
+        <v>105</v>
       </c>
       <c r="C35" t="s">
-        <v>214</v>
+        <v>166</v>
       </c>
       <c r="D35">
-        <v>50.61273699999999</v>
+        <v>49.7097598</v>
       </c>
       <c r="E35">
-        <v>3.123373</v>
+        <v>2.773197300000001</v>
       </c>
       <c r="F35">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="G35">
-        <v>4178</v>
+        <v>1068</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -2653,10 +2350,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>302</v>
+        <v>229</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2664,34 +2361,34 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="C36" t="s">
-        <v>215</v>
+        <v>167</v>
       </c>
       <c r="D36">
-        <v>50.6427316</v>
+        <v>49.8708087</v>
       </c>
       <c r="E36">
-        <v>3.0668892</v>
+        <v>2.5975248</v>
       </c>
       <c r="F36">
         <v>4.5</v>
       </c>
       <c r="G36">
-        <v>4716</v>
+        <v>169</v>
       </c>
       <c r="H36">
         <v>2</v>
       </c>
       <c r="I36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>303</v>
+        <v>230</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2699,31 +2396,34 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="C37" t="s">
-        <v>216</v>
+        <v>168</v>
       </c>
       <c r="D37">
-        <v>50.43022910000001</v>
+        <v>49.7089958</v>
       </c>
       <c r="E37">
-        <v>2.8241761</v>
+        <v>2.773895500000001</v>
       </c>
       <c r="F37">
-        <v>4.6</v>
+        <v>3.8</v>
       </c>
       <c r="G37">
-        <v>429</v>
+        <v>831</v>
+      </c>
+      <c r="H37">
+        <v>2</v>
       </c>
       <c r="I37" t="b">
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>268</v>
+        <v>194</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>304</v>
+        <v>231</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2731,22 +2431,22 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="C38" t="s">
-        <v>217</v>
+        <v>169</v>
       </c>
       <c r="D38">
-        <v>50.42831</v>
+        <v>49.6995639</v>
       </c>
       <c r="E38">
-        <v>2.826468599999999</v>
+        <v>2.7944886</v>
       </c>
       <c r="F38">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="G38">
-        <v>847</v>
+        <v>175</v>
       </c>
       <c r="H38">
         <v>2</v>
@@ -2755,10 +2455,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>268</v>
+        <v>194</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>305</v>
+        <v>232</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2766,34 +2466,34 @@
         <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>133</v>
+        <v>109</v>
       </c>
       <c r="C39" t="s">
-        <v>218</v>
+        <v>170</v>
       </c>
       <c r="D39">
-        <v>50.2927725</v>
+        <v>50.1980106</v>
       </c>
       <c r="E39">
-        <v>2.780148199999999</v>
+        <v>2.8759627</v>
       </c>
       <c r="F39">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="G39">
-        <v>690</v>
+        <v>82</v>
       </c>
       <c r="H39">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>268</v>
+        <v>194</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>306</v>
+        <v>233</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2801,28 +2501,31 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>134</v>
+        <v>110</v>
       </c>
       <c r="C40" t="s">
-        <v>219</v>
+        <v>171</v>
       </c>
       <c r="D40">
-        <v>50.3472046</v>
+        <v>49.6978505</v>
       </c>
       <c r="E40">
-        <v>2.6535711</v>
+        <v>2.791623399999999</v>
       </c>
       <c r="F40">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="G40">
-        <v>163</v>
+        <v>201</v>
+      </c>
+      <c r="I40" t="b">
+        <v>1</v>
       </c>
       <c r="J40" t="s">
-        <v>268</v>
+        <v>194</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>307</v>
+        <v>234</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2830,34 +2533,31 @@
         <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>135</v>
+        <v>111</v>
       </c>
       <c r="C41" t="s">
-        <v>220</v>
+        <v>172</v>
       </c>
       <c r="D41">
-        <v>50.4796752</v>
+        <v>50.17135099999999</v>
       </c>
       <c r="E41">
-        <v>3.237034299999999</v>
+        <v>2.6318673</v>
       </c>
       <c r="F41">
-        <v>4.5</v>
+        <v>4.9</v>
       </c>
       <c r="G41">
-        <v>473</v>
-      </c>
-      <c r="H41">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="I41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>308</v>
+        <v>235</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2865,34 +2565,31 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="C42" t="s">
-        <v>221</v>
+        <v>173</v>
       </c>
       <c r="D42">
-        <v>50.367342</v>
+        <v>50.0034562</v>
       </c>
       <c r="E42">
-        <v>3.081729999999999</v>
+        <v>2.911265</v>
       </c>
       <c r="F42">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="G42">
-        <v>376</v>
-      </c>
-      <c r="H42">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>309</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2900,34 +2597,34 @@
         <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>137</v>
+        <v>113</v>
       </c>
       <c r="C43" t="s">
-        <v>222</v>
+        <v>174</v>
       </c>
       <c r="D43">
-        <v>50.3691968</v>
+        <v>49.6905687</v>
       </c>
       <c r="E43">
-        <v>3.078329</v>
+        <v>2.788442</v>
       </c>
       <c r="F43">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
       <c r="G43">
-        <v>464</v>
+        <v>221</v>
       </c>
       <c r="H43">
         <v>2</v>
       </c>
       <c r="I43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>310</v>
+        <v>237</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2935,34 +2632,31 @@
         <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="C44" t="s">
-        <v>223</v>
+        <v>175</v>
       </c>
       <c r="D44">
-        <v>50.2091985</v>
+        <v>49.7447927</v>
       </c>
       <c r="E44">
-        <v>3.1905208</v>
+        <v>3.0752862</v>
       </c>
       <c r="F44">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="G44">
-        <v>398</v>
-      </c>
-      <c r="H44">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="I44" t="b">
         <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>311</v>
+        <v>238</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2970,22 +2664,22 @@
         <v>54</v>
       </c>
       <c r="B45" t="s">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="C45" t="s">
-        <v>224</v>
+        <v>176</v>
       </c>
       <c r="D45">
-        <v>50.0990133</v>
+        <v>49.35251799999999</v>
       </c>
       <c r="E45">
-        <v>2.8551931</v>
+        <v>2.767293</v>
       </c>
       <c r="F45">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="G45">
-        <v>888</v>
+        <v>1252</v>
       </c>
       <c r="H45">
         <v>2</v>
@@ -2994,10 +2688,10 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>312</v>
+        <v>239</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -3005,34 +2699,34 @@
         <v>55</v>
       </c>
       <c r="B46" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="C46" t="s">
-        <v>225</v>
+        <v>177</v>
       </c>
       <c r="D46">
-        <v>50.0440674</v>
+        <v>49.64668830000001</v>
       </c>
       <c r="E46">
-        <v>2.666995500000001</v>
+        <v>2.56774</v>
       </c>
       <c r="F46">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="G46">
-        <v>606</v>
+        <v>401</v>
       </c>
       <c r="H46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I46" t="b">
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>313</v>
+        <v>240</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -3040,34 +2734,31 @@
         <v>56</v>
       </c>
       <c r="B47" t="s">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="C47" t="s">
-        <v>226</v>
+        <v>178</v>
       </c>
       <c r="D47">
-        <v>49.9306446</v>
+        <v>49.2062605</v>
       </c>
       <c r="E47">
-        <v>2.9373479</v>
+        <v>2.5796583</v>
       </c>
       <c r="F47">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="G47">
-        <v>687</v>
-      </c>
-      <c r="H47">
-        <v>2</v>
+        <v>321</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>314</v>
+        <v>241</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -3075,34 +2766,34 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="C48" t="s">
-        <v>227</v>
+        <v>179</v>
       </c>
       <c r="D48">
-        <v>49.9294497</v>
+        <v>49.32945489999999</v>
       </c>
       <c r="E48">
-        <v>2.9385445</v>
+        <v>2.465046000000001</v>
       </c>
       <c r="F48">
-        <v>4.7</v>
+        <v>3.7</v>
       </c>
       <c r="G48">
-        <v>340</v>
+        <v>141</v>
       </c>
       <c r="H48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I48" t="b">
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>315</v>
+        <v>242</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -3110,31 +2801,34 @@
         <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="C49" t="s">
-        <v>228</v>
+        <v>180</v>
       </c>
       <c r="D49">
-        <v>49.887574</v>
+        <v>49.32898950000001</v>
       </c>
       <c r="E49">
-        <v>2.837822</v>
+        <v>2.4629503</v>
       </c>
       <c r="F49">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="G49">
-        <v>627</v>
+        <v>616</v>
+      </c>
+      <c r="H49">
+        <v>1</v>
       </c>
       <c r="I49" t="b">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>316</v>
+        <v>243</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3142,31 +2836,34 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>144</v>
+        <v>120</v>
       </c>
       <c r="C50" t="s">
-        <v>229</v>
+        <v>181</v>
       </c>
       <c r="D50">
-        <v>49.9157805</v>
+        <v>49.4786609</v>
       </c>
       <c r="E50">
-        <v>2.9340714</v>
+        <v>2.8784628</v>
       </c>
       <c r="F50">
         <v>4.4</v>
       </c>
       <c r="G50">
-        <v>138</v>
+        <v>545</v>
+      </c>
+      <c r="H50">
+        <v>2</v>
       </c>
       <c r="I50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>317</v>
+        <v>244</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3174,34 +2871,34 @@
         <v>60</v>
       </c>
       <c r="B51" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="C51" t="s">
-        <v>230</v>
+        <v>182</v>
       </c>
       <c r="D51">
-        <v>49.812285</v>
+        <v>49.3854719</v>
       </c>
       <c r="E51">
-        <v>2.7008719</v>
+        <v>2.777325000000001</v>
       </c>
       <c r="F51">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="G51">
-        <v>90</v>
+        <v>777</v>
       </c>
       <c r="H51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>318</v>
+        <v>245</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3209,34 +2906,31 @@
         <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>146</v>
+        <v>122</v>
       </c>
       <c r="C52" t="s">
-        <v>231</v>
+        <v>183</v>
       </c>
       <c r="D52">
-        <v>49.9470246</v>
+        <v>49.398555</v>
       </c>
       <c r="E52">
-        <v>3.1002615</v>
+        <v>2.7974006</v>
       </c>
       <c r="F52">
-        <v>4.6</v>
+        <v>4.1</v>
       </c>
       <c r="G52">
-        <v>183</v>
-      </c>
-      <c r="H52">
-        <v>2</v>
+        <v>117</v>
       </c>
       <c r="I52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>319</v>
+        <v>246</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -3244,34 +2938,34 @@
         <v>62</v>
       </c>
       <c r="B53" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" t="s">
+        <v>184</v>
+      </c>
+      <c r="D53">
+        <v>49.551745</v>
+      </c>
+      <c r="E53">
+        <v>2.520455</v>
+      </c>
+      <c r="F53">
+        <v>4.6</v>
+      </c>
+      <c r="G53">
         <v>147</v>
       </c>
-      <c r="C53" t="s">
-        <v>232</v>
-      </c>
-      <c r="D53">
-        <v>49.9000698</v>
-      </c>
-      <c r="E53">
-        <v>2.5028801</v>
-      </c>
-      <c r="F53">
-        <v>4.5</v>
-      </c>
-      <c r="G53">
-        <v>223</v>
-      </c>
       <c r="H53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>320</v>
+        <v>247</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -3279,34 +2973,34 @@
         <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>148</v>
+        <v>124</v>
       </c>
       <c r="C54" t="s">
-        <v>233</v>
+        <v>185</v>
       </c>
       <c r="D54">
-        <v>50.0409911</v>
+        <v>49.3084</v>
       </c>
       <c r="E54">
-        <v>2.6686785</v>
+        <v>2.728939</v>
       </c>
       <c r="F54">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="G54">
-        <v>581</v>
+        <v>460</v>
       </c>
       <c r="H54">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>321</v>
+        <v>248</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -3314,34 +3008,31 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>149</v>
+        <v>125</v>
       </c>
       <c r="C55" t="s">
-        <v>234</v>
+        <v>186</v>
       </c>
       <c r="D55">
-        <v>49.9291968</v>
+        <v>49.4260495</v>
       </c>
       <c r="E55">
-        <v>2.933116499999999</v>
+        <v>2.6380979</v>
       </c>
       <c r="F55">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="G55">
-        <v>911</v>
-      </c>
-      <c r="H55">
-        <v>2</v>
+        <v>209</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>322</v>
+        <v>249</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -3349,34 +3040,34 @@
         <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
       <c r="C56" t="s">
-        <v>235</v>
+        <v>187</v>
       </c>
       <c r="D56">
-        <v>49.7097598</v>
+        <v>49.4888858</v>
       </c>
       <c r="E56">
-        <v>2.773197300000001</v>
+        <v>2.8153957</v>
       </c>
       <c r="F56">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="G56">
-        <v>1068</v>
+        <v>142</v>
       </c>
       <c r="H56">
         <v>2</v>
       </c>
       <c r="I56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J56" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>323</v>
+        <v>250</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -3384,34 +3075,34 @@
         <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>151</v>
+        <v>127</v>
       </c>
       <c r="C57" t="s">
-        <v>236</v>
+        <v>188</v>
       </c>
       <c r="D57">
-        <v>49.8708087</v>
+        <v>49.4291534</v>
       </c>
       <c r="E57">
-        <v>2.5975248</v>
+        <v>2.8386883</v>
       </c>
       <c r="F57">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="G57">
-        <v>169</v>
+        <v>81</v>
       </c>
       <c r="H57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J57" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>324</v>
+        <v>251</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -3419,34 +3110,31 @@
         <v>67</v>
       </c>
       <c r="B58" t="s">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="C58" t="s">
-        <v>237</v>
+        <v>189</v>
       </c>
       <c r="D58">
-        <v>49.7089958</v>
+        <v>49.4219351</v>
       </c>
       <c r="E58">
-        <v>2.773895500000001</v>
+        <v>2.8431248</v>
       </c>
       <c r="F58">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="G58">
-        <v>831</v>
+        <v>197</v>
       </c>
       <c r="H58">
-        <v>2</v>
-      </c>
-      <c r="I58" t="b">
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>325</v>
+        <v>252</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -3454,34 +3142,31 @@
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>153</v>
+        <v>129</v>
       </c>
       <c r="C59" t="s">
-        <v>238</v>
+        <v>190</v>
       </c>
       <c r="D59">
-        <v>49.6995639</v>
+        <v>49.416086</v>
       </c>
       <c r="E59">
-        <v>2.7944886</v>
+        <v>2.819035</v>
       </c>
       <c r="F59">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="G59">
-        <v>175</v>
-      </c>
-      <c r="H59">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>326</v>
+        <v>253</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -3489,34 +3174,34 @@
         <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="C60" t="s">
-        <v>239</v>
+        <v>191</v>
       </c>
       <c r="D60">
-        <v>50.1980106</v>
+        <v>49.4057464</v>
       </c>
       <c r="E60">
-        <v>2.8759627</v>
+        <v>2.7834179</v>
       </c>
       <c r="F60">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="G60">
-        <v>82</v>
+        <v>4050</v>
       </c>
       <c r="H60">
         <v>1</v>
       </c>
       <c r="I60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>327</v>
+        <v>254</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -3524,31 +3209,34 @@
         <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>155</v>
+        <v>131</v>
       </c>
       <c r="C61" t="s">
-        <v>240</v>
+        <v>192</v>
       </c>
       <c r="D61">
-        <v>49.6978505</v>
+        <v>49.4054683</v>
       </c>
       <c r="E61">
-        <v>2.791623399999999</v>
+        <v>2.7843017</v>
       </c>
       <c r="F61">
-        <v>4.6</v>
+        <v>4.1</v>
       </c>
       <c r="G61">
-        <v>201</v>
+        <v>5360</v>
+      </c>
+      <c r="H61">
+        <v>2</v>
       </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>328</v>
+        <v>255</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -3556,850 +3244,34 @@
         <v>71</v>
       </c>
       <c r="B62" t="s">
-        <v>156</v>
+        <v>132</v>
       </c>
       <c r="C62" t="s">
-        <v>241</v>
+        <v>193</v>
       </c>
       <c r="D62">
-        <v>50.17135099999999</v>
+        <v>49.39665679999999</v>
       </c>
       <c r="E62">
-        <v>2.6318673</v>
+        <v>2.786974299999999</v>
       </c>
       <c r="F62">
-        <v>4.9</v>
+        <v>3.9</v>
       </c>
       <c r="G62">
-        <v>49</v>
+        <v>154</v>
+      </c>
+      <c r="H62">
+        <v>2</v>
       </c>
       <c r="I62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>266</v>
+        <v>194</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11">
-      <c r="A63" t="s">
-        <v>72</v>
-      </c>
-      <c r="B63" t="s">
-        <v>157</v>
-      </c>
-      <c r="C63" t="s">
-        <v>242</v>
-      </c>
-      <c r="D63">
-        <v>50.0034562</v>
-      </c>
-      <c r="E63">
-        <v>2.911265</v>
-      </c>
-      <c r="F63">
-        <v>3.5</v>
-      </c>
-      <c r="G63">
-        <v>11</v>
-      </c>
-      <c r="I63" t="b">
-        <v>0</v>
-      </c>
-      <c r="J63" t="s">
-        <v>266</v>
-      </c>
-      <c r="K63" s="2" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11">
-      <c r="A64" t="s">
-        <v>73</v>
-      </c>
-      <c r="B64" t="s">
-        <v>158</v>
-      </c>
-      <c r="C64" t="s">
-        <v>243</v>
-      </c>
-      <c r="D64">
-        <v>49.6905687</v>
-      </c>
-      <c r="E64">
-        <v>2.788442</v>
-      </c>
-      <c r="F64">
-        <v>3.9</v>
-      </c>
-      <c r="G64">
-        <v>221</v>
-      </c>
-      <c r="H64">
-        <v>2</v>
-      </c>
-      <c r="I64" t="b">
-        <v>0</v>
-      </c>
-      <c r="J64" t="s">
-        <v>266</v>
-      </c>
-      <c r="K64" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11">
-      <c r="A65" t="s">
-        <v>74</v>
-      </c>
-      <c r="B65" t="s">
-        <v>159</v>
-      </c>
-      <c r="C65" t="s">
-        <v>244</v>
-      </c>
-      <c r="D65">
-        <v>49.7447927</v>
-      </c>
-      <c r="E65">
-        <v>3.0752862</v>
-      </c>
-      <c r="F65">
-        <v>4.1</v>
-      </c>
-      <c r="G65">
-        <v>58</v>
-      </c>
-      <c r="I65" t="b">
-        <v>1</v>
-      </c>
-      <c r="J65" t="s">
-        <v>266</v>
-      </c>
-      <c r="K65" s="2" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11">
-      <c r="A66" t="s">
-        <v>75</v>
-      </c>
-      <c r="B66" t="s">
-        <v>160</v>
-      </c>
-      <c r="C66" t="s">
-        <v>245</v>
-      </c>
-      <c r="D66">
-        <v>49.41652569999999</v>
-      </c>
-      <c r="E66">
-        <v>2.8255822</v>
-      </c>
-      <c r="F66">
-        <v>4.5</v>
-      </c>
-      <c r="G66">
-        <v>367</v>
-      </c>
-      <c r="H66">
-        <v>2</v>
-      </c>
-      <c r="I66" t="b">
-        <v>1</v>
-      </c>
-      <c r="J66" t="s">
-        <v>266</v>
-      </c>
-      <c r="K66" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11">
-      <c r="A67" t="s">
-        <v>76</v>
-      </c>
-      <c r="B67" t="s">
-        <v>161</v>
-      </c>
-      <c r="C67" t="s">
-        <v>246</v>
-      </c>
-      <c r="D67">
-        <v>49.35251799999999</v>
-      </c>
-      <c r="E67">
-        <v>2.767293</v>
-      </c>
-      <c r="F67">
-        <v>4.8</v>
-      </c>
-      <c r="G67">
-        <v>1247</v>
-      </c>
-      <c r="H67">
-        <v>2</v>
-      </c>
-      <c r="I67" t="b">
-        <v>1</v>
-      </c>
-      <c r="J67" t="s">
-        <v>266</v>
-      </c>
-      <c r="K67" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11">
-      <c r="A68" t="s">
-        <v>77</v>
-      </c>
-      <c r="B68" t="s">
-        <v>162</v>
-      </c>
-      <c r="C68" t="s">
-        <v>247</v>
-      </c>
-      <c r="D68">
-        <v>49.64668830000001</v>
-      </c>
-      <c r="E68">
-        <v>2.56774</v>
-      </c>
-      <c r="F68">
-        <v>4.4</v>
-      </c>
-      <c r="G68">
-        <v>401</v>
-      </c>
-      <c r="H68">
-        <v>1</v>
-      </c>
-      <c r="I68" t="b">
-        <v>1</v>
-      </c>
-      <c r="J68" t="s">
-        <v>266</v>
-      </c>
-      <c r="K68" s="2" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11">
-      <c r="A69" t="s">
-        <v>78</v>
-      </c>
-      <c r="B69" t="s">
-        <v>163</v>
-      </c>
-      <c r="C69" t="s">
-        <v>248</v>
-      </c>
-      <c r="D69">
-        <v>49.4181602</v>
-      </c>
-      <c r="E69">
-        <v>2.8260746</v>
-      </c>
-      <c r="F69">
-        <v>4.3</v>
-      </c>
-      <c r="G69">
-        <v>95</v>
-      </c>
-      <c r="H69">
-        <v>2</v>
-      </c>
-      <c r="I69" t="b">
-        <v>1</v>
-      </c>
-      <c r="J69" t="s">
-        <v>266</v>
-      </c>
-      <c r="K69" s="2" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11">
-      <c r="A70" t="s">
-        <v>79</v>
-      </c>
-      <c r="B70" t="s">
-        <v>164</v>
-      </c>
-      <c r="C70" t="s">
-        <v>249</v>
-      </c>
-      <c r="D70">
-        <v>49.2062605</v>
-      </c>
-      <c r="E70">
-        <v>2.5796583</v>
-      </c>
-      <c r="F70">
-        <v>4.6</v>
-      </c>
-      <c r="G70">
-        <v>321</v>
-      </c>
-      <c r="I70" t="b">
-        <v>1</v>
-      </c>
-      <c r="J70" t="s">
-        <v>266</v>
-      </c>
-      <c r="K70" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11">
-      <c r="A71" t="s">
-        <v>80</v>
-      </c>
-      <c r="B71" t="s">
-        <v>165</v>
-      </c>
-      <c r="C71" t="s">
-        <v>250</v>
-      </c>
-      <c r="D71">
-        <v>49.32945489999999</v>
-      </c>
-      <c r="E71">
-        <v>2.465046000000001</v>
-      </c>
-      <c r="F71">
-        <v>3.7</v>
-      </c>
-      <c r="G71">
-        <v>140</v>
-      </c>
-      <c r="H71">
-        <v>1</v>
-      </c>
-      <c r="I71" t="b">
-        <v>1</v>
-      </c>
-      <c r="J71" t="s">
-        <v>266</v>
-      </c>
-      <c r="K71" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11">
-      <c r="A72" t="s">
-        <v>81</v>
-      </c>
-      <c r="B72" t="s">
-        <v>166</v>
-      </c>
-      <c r="C72" t="s">
-        <v>251</v>
-      </c>
-      <c r="D72">
-        <v>49.32898950000001</v>
-      </c>
-      <c r="E72">
-        <v>2.4629503</v>
-      </c>
-      <c r="F72">
-        <v>4.6</v>
-      </c>
-      <c r="G72">
-        <v>616</v>
-      </c>
-      <c r="H72">
-        <v>1</v>
-      </c>
-      <c r="I72" t="b">
-        <v>1</v>
-      </c>
-      <c r="J72" t="s">
-        <v>268</v>
-      </c>
-      <c r="K72" s="2" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11">
-      <c r="A73" t="s">
-        <v>82</v>
-      </c>
-      <c r="B73" t="s">
-        <v>167</v>
-      </c>
-      <c r="C73" t="s">
-        <v>252</v>
-      </c>
-      <c r="D73">
-        <v>49.4786609</v>
-      </c>
-      <c r="E73">
-        <v>2.8784628</v>
-      </c>
-      <c r="F73">
-        <v>4.4</v>
-      </c>
-      <c r="G73">
-        <v>545</v>
-      </c>
-      <c r="H73">
-        <v>2</v>
-      </c>
-      <c r="I73" t="b">
-        <v>1</v>
-      </c>
-      <c r="J73" t="s">
-        <v>268</v>
-      </c>
-      <c r="K73" s="2" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11">
-      <c r="A74" t="s">
-        <v>83</v>
-      </c>
-      <c r="B74" t="s">
-        <v>168</v>
-      </c>
-      <c r="C74" t="s">
-        <v>253</v>
-      </c>
-      <c r="D74">
-        <v>49.3854719</v>
-      </c>
-      <c r="E74">
-        <v>2.777325000000001</v>
-      </c>
-      <c r="F74">
-        <v>4.5</v>
-      </c>
-      <c r="G74">
-        <v>777</v>
-      </c>
-      <c r="H74">
-        <v>2</v>
-      </c>
-      <c r="I74" t="b">
-        <v>1</v>
-      </c>
-      <c r="J74" t="s">
-        <v>268</v>
-      </c>
-      <c r="K74" s="2" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11">
-      <c r="A75" t="s">
-        <v>84</v>
-      </c>
-      <c r="B75" t="s">
-        <v>169</v>
-      </c>
-      <c r="C75" t="s">
-        <v>254</v>
-      </c>
-      <c r="D75">
-        <v>49.398555</v>
-      </c>
-      <c r="E75">
-        <v>2.7974006</v>
-      </c>
-      <c r="F75">
-        <v>4.1</v>
-      </c>
-      <c r="G75">
-        <v>117</v>
-      </c>
-      <c r="I75" t="b">
-        <v>1</v>
-      </c>
-      <c r="J75" t="s">
-        <v>268</v>
-      </c>
-      <c r="K75" s="2" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11">
-      <c r="A76" t="s">
-        <v>85</v>
-      </c>
-      <c r="B76" t="s">
-        <v>170</v>
-      </c>
-      <c r="C76" t="s">
-        <v>255</v>
-      </c>
-      <c r="D76">
-        <v>49.551745</v>
-      </c>
-      <c r="E76">
-        <v>2.520455</v>
-      </c>
-      <c r="F76">
-        <v>4.6</v>
-      </c>
-      <c r="G76">
-        <v>147</v>
-      </c>
-      <c r="H76">
-        <v>1</v>
-      </c>
-      <c r="I76" t="b">
-        <v>1</v>
-      </c>
-      <c r="J76" t="s">
-        <v>268</v>
-      </c>
-      <c r="K76" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11">
-      <c r="A77" t="s">
-        <v>86</v>
-      </c>
-      <c r="B77" t="s">
-        <v>171</v>
-      </c>
-      <c r="C77" t="s">
         <v>256</v>
-      </c>
-      <c r="D77">
-        <v>49.3084</v>
-      </c>
-      <c r="E77">
-        <v>2.728939</v>
-      </c>
-      <c r="F77">
-        <v>4.4</v>
-      </c>
-      <c r="G77">
-        <v>460</v>
-      </c>
-      <c r="H77">
-        <v>1</v>
-      </c>
-      <c r="I77" t="b">
-        <v>1</v>
-      </c>
-      <c r="J77" t="s">
-        <v>268</v>
-      </c>
-      <c r="K77" s="2" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11">
-      <c r="A78" t="s">
-        <v>87</v>
-      </c>
-      <c r="B78" t="s">
-        <v>172</v>
-      </c>
-      <c r="C78" t="s">
-        <v>257</v>
-      </c>
-      <c r="D78">
-        <v>49.4260495</v>
-      </c>
-      <c r="E78">
-        <v>2.6380979</v>
-      </c>
-      <c r="F78">
-        <v>4.4</v>
-      </c>
-      <c r="G78">
-        <v>209</v>
-      </c>
-      <c r="I78" t="b">
-        <v>1</v>
-      </c>
-      <c r="J78" t="s">
-        <v>268</v>
-      </c>
-      <c r="K78" s="2" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11">
-      <c r="A79" t="s">
-        <v>88</v>
-      </c>
-      <c r="B79" t="s">
-        <v>173</v>
-      </c>
-      <c r="C79" t="s">
-        <v>258</v>
-      </c>
-      <c r="D79">
-        <v>49.4171323</v>
-      </c>
-      <c r="E79">
-        <v>2.826151</v>
-      </c>
-      <c r="F79">
-        <v>4</v>
-      </c>
-      <c r="G79">
-        <v>1419</v>
-      </c>
-      <c r="H79">
-        <v>2</v>
-      </c>
-      <c r="I79" t="b">
-        <v>1</v>
-      </c>
-      <c r="J79" t="s">
-        <v>268</v>
-      </c>
-      <c r="K79" s="2" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11">
-      <c r="A80" t="s">
-        <v>89</v>
-      </c>
-      <c r="B80" t="s">
-        <v>174</v>
-      </c>
-      <c r="C80" t="s">
-        <v>259</v>
-      </c>
-      <c r="D80">
-        <v>49.4888858</v>
-      </c>
-      <c r="E80">
-        <v>2.8153957</v>
-      </c>
-      <c r="F80">
-        <v>4.4</v>
-      </c>
-      <c r="G80">
-        <v>142</v>
-      </c>
-      <c r="H80">
-        <v>2</v>
-      </c>
-      <c r="I80" t="b">
-        <v>1</v>
-      </c>
-      <c r="J80" t="s">
-        <v>268</v>
-      </c>
-      <c r="K80" s="2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11">
-      <c r="A81" t="s">
-        <v>90</v>
-      </c>
-      <c r="B81" t="s">
-        <v>175</v>
-      </c>
-      <c r="C81" t="s">
-        <v>260</v>
-      </c>
-      <c r="D81">
-        <v>49.4291534</v>
-      </c>
-      <c r="E81">
-        <v>2.8386883</v>
-      </c>
-      <c r="F81">
-        <v>4.3</v>
-      </c>
-      <c r="G81">
-        <v>81</v>
-      </c>
-      <c r="H81">
-        <v>1</v>
-      </c>
-      <c r="I81" t="b">
-        <v>0</v>
-      </c>
-      <c r="J81" t="s">
-        <v>268</v>
-      </c>
-      <c r="K81" s="2" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11">
-      <c r="A82" t="s">
-        <v>91</v>
-      </c>
-      <c r="B82" t="s">
-        <v>176</v>
-      </c>
-      <c r="C82" t="s">
-        <v>261</v>
-      </c>
-      <c r="D82">
-        <v>49.4219351</v>
-      </c>
-      <c r="E82">
-        <v>2.8431248</v>
-      </c>
-      <c r="F82">
-        <v>4.4</v>
-      </c>
-      <c r="G82">
-        <v>197</v>
-      </c>
-      <c r="H82">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
-        <v>268</v>
-      </c>
-      <c r="K82" s="2" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11">
-      <c r="A83" t="s">
-        <v>92</v>
-      </c>
-      <c r="B83" t="s">
-        <v>177</v>
-      </c>
-      <c r="C83" t="s">
-        <v>262</v>
-      </c>
-      <c r="D83">
-        <v>49.416086</v>
-      </c>
-      <c r="E83">
-        <v>2.819035</v>
-      </c>
-      <c r="F83">
-        <v>4.2</v>
-      </c>
-      <c r="G83">
-        <v>114</v>
-      </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
-        <v>268</v>
-      </c>
-      <c r="K83" s="2" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11">
-      <c r="A84" t="s">
-        <v>93</v>
-      </c>
-      <c r="B84" t="s">
-        <v>178</v>
-      </c>
-      <c r="C84" t="s">
-        <v>263</v>
-      </c>
-      <c r="D84">
-        <v>49.4057464</v>
-      </c>
-      <c r="E84">
-        <v>2.7834179</v>
-      </c>
-      <c r="F84">
-        <v>4.2</v>
-      </c>
-      <c r="G84">
-        <v>4038</v>
-      </c>
-      <c r="H84">
-        <v>1</v>
-      </c>
-      <c r="I84" t="b">
-        <v>1</v>
-      </c>
-      <c r="J84" t="s">
-        <v>268</v>
-      </c>
-      <c r="K84" s="2" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11">
-      <c r="A85" t="s">
-        <v>94</v>
-      </c>
-      <c r="B85" t="s">
-        <v>179</v>
-      </c>
-      <c r="C85" t="s">
-        <v>264</v>
-      </c>
-      <c r="D85">
-        <v>49.4054683</v>
-      </c>
-      <c r="E85">
-        <v>2.7843017</v>
-      </c>
-      <c r="F85">
-        <v>4.1</v>
-      </c>
-      <c r="G85">
-        <v>5356</v>
-      </c>
-      <c r="H85">
-        <v>2</v>
-      </c>
-      <c r="I85" t="b">
-        <v>1</v>
-      </c>
-      <c r="J85" t="s">
-        <v>268</v>
-      </c>
-      <c r="K85" s="2" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11">
-      <c r="A86" t="s">
-        <v>95</v>
-      </c>
-      <c r="B86" t="s">
-        <v>180</v>
-      </c>
-      <c r="C86" t="s">
-        <v>265</v>
-      </c>
-      <c r="D86">
-        <v>49.39665679999999</v>
-      </c>
-      <c r="E86">
-        <v>2.786974299999999</v>
-      </c>
-      <c r="F86">
-        <v>3.9</v>
-      </c>
-      <c r="G86">
-        <v>154</v>
-      </c>
-      <c r="H86">
-        <v>2</v>
-      </c>
-      <c r="I86" t="b">
-        <v>1</v>
-      </c>
-      <c r="J86" t="s">
-        <v>268</v>
-      </c>
-      <c r="K86" s="2" t="s">
-        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -4465,30 +3337,6 @@
     <hyperlink ref="K60" r:id="rId59"/>
     <hyperlink ref="K61" r:id="rId60"/>
     <hyperlink ref="K62" r:id="rId61"/>
-    <hyperlink ref="K63" r:id="rId62"/>
-    <hyperlink ref="K64" r:id="rId63"/>
-    <hyperlink ref="K65" r:id="rId64"/>
-    <hyperlink ref="K66" r:id="rId65"/>
-    <hyperlink ref="K67" r:id="rId66"/>
-    <hyperlink ref="K68" r:id="rId67"/>
-    <hyperlink ref="K69" r:id="rId68"/>
-    <hyperlink ref="K70" r:id="rId69"/>
-    <hyperlink ref="K71" r:id="rId70"/>
-    <hyperlink ref="K72" r:id="rId71"/>
-    <hyperlink ref="K73" r:id="rId72"/>
-    <hyperlink ref="K74" r:id="rId73"/>
-    <hyperlink ref="K75" r:id="rId74"/>
-    <hyperlink ref="K76" r:id="rId75"/>
-    <hyperlink ref="K77" r:id="rId76"/>
-    <hyperlink ref="K78" r:id="rId77"/>
-    <hyperlink ref="K79" r:id="rId78"/>
-    <hyperlink ref="K80" r:id="rId79"/>
-    <hyperlink ref="K81" r:id="rId80"/>
-    <hyperlink ref="K82" r:id="rId81"/>
-    <hyperlink ref="K83" r:id="rId82"/>
-    <hyperlink ref="K84" r:id="rId83"/>
-    <hyperlink ref="K85" r:id="rId84"/>
-    <hyperlink ref="K86" r:id="rId85"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>